<commit_message>
Change pixel cycles from 3797 to 3801
</commit_message>
<xml_diff>
--- a/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
+++ b/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE45E75-8A94-4E09-A299-DAE840449EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3FC44E-CB62-42CC-853C-55730C589838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3825" yWindow="2843" windowWidth="24157" windowHeight="15202" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="18676" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="60">
   <si>
     <t>SM0</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -153,10 +153,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>45636 ticks each scan row (exclude expsorure delay)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>time per frame (ms)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -169,10 +165,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>1/2730.45</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>1/2000.1280</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -209,18 +201,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>MSB pixel 3792</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>LSB pixel 3791</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>MSB pixel 3791</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>~41MiB/s</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -246,6 +226,38 @@
   </si>
   <si>
     <t>exposure ticks</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MSB pixel 3795</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>LSB pixel 3795</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MSB pixel 3796</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>45684 ticks each scan row (exclude expsorure delay)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/2728.30</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>~24MiB/s</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>~18MiB/s</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>~15MiB/s</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -503,13 +515,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -852,13 +864,13 @@
   <sheetData>
     <row r="1" spans="1:14" ht="27.75" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -873,7 +885,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.4">
@@ -912,14 +924,14 @@
         <v>30</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>-16</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="1"/>
@@ -930,10 +942,10 @@
       <c r="A6">
         <v>-15</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="21"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -941,34 +953,34 @@
       <c r="A7">
         <v>-14</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="21"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="20"/>
+      <c r="G7" s="19"/>
       <c r="J7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s">
         <v>32</v>
       </c>
       <c r="L7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" t="s">
         <v>34</v>
       </c>
-      <c r="M7" t="s">
-        <v>35</v>
-      </c>
       <c r="N7" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>-13</v>
       </c>
-      <c r="D8" s="19"/>
+      <c r="D8" s="21"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="20"/>
+      <c r="G8" s="19"/>
       <c r="J8" s="17">
         <v>0</v>
       </c>
@@ -979,45 +991,45 @@
         <v>0.36518400000000001</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>-12</v>
       </c>
-      <c r="D9" s="19"/>
+      <c r="D9" s="21"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="20" t="s">
         <v>5</v>
       </c>
       <c r="J9">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K9">
-        <v>45780</v>
+        <v>45828</v>
       </c>
       <c r="L9">
-        <v>0.36624000000000001</v>
+        <v>0.36652800000000002</v>
       </c>
       <c r="M9" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>-11</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="21"/>
+      <c r="G10" s="20"/>
       <c r="J10">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="K10">
         <v>50004</v>
@@ -1026,22 +1038,22 @@
         <v>0.400032</v>
       </c>
       <c r="M10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="N10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>-10</v>
       </c>
-      <c r="D11" s="19"/>
+      <c r="D11" s="21"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="21"/>
+      <c r="G11" s="20"/>
       <c r="J11">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="K11">
         <v>62496</v>
@@ -1050,24 +1062,24 @@
         <v>0.49996800000000002</v>
       </c>
       <c r="M11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="N11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>-9</v>
       </c>
-      <c r="D12" s="19"/>
+      <c r="D12" s="21"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="19" t="s">
         <v>6</v>
       </c>
       <c r="J12">
-        <v>2706</v>
+        <v>2702</v>
       </c>
       <c r="K12">
         <v>78120</v>
@@ -1076,19 +1088,22 @@
         <v>0.62495999999999996</v>
       </c>
       <c r="M12" t="s">
-        <v>42</v>
+        <v>40</v>
+      </c>
+      <c r="N12" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>-8</v>
       </c>
-      <c r="D13" s="19"/>
+      <c r="D13" s="21"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="20"/>
+      <c r="G13" s="19"/>
       <c r="J13">
-        <v>4529</v>
+        <v>4525</v>
       </c>
       <c r="K13">
         <v>99996</v>
@@ -1097,19 +1112,22 @@
         <v>0.79996800000000001</v>
       </c>
       <c r="M13" t="s">
-        <v>41</v>
+        <v>39</v>
+      </c>
+      <c r="N13" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>-7</v>
       </c>
-      <c r="D14" s="19"/>
+      <c r="D14" s="21"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="20"/>
+      <c r="G14" s="19"/>
       <c r="J14">
-        <v>6613</v>
+        <v>6609</v>
       </c>
       <c r="K14">
         <v>125004</v>
@@ -1118,17 +1136,20 @@
         <v>1.000032</v>
       </c>
       <c r="M14" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="N14" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>-6</v>
       </c>
-      <c r="D15" s="19"/>
+      <c r="D15" s="21"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="21" t="s">
+      <c r="G15" s="20" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1136,28 +1157,28 @@
       <c r="A16">
         <v>-5</v>
       </c>
-      <c r="D16" s="19"/>
+      <c r="D16" s="21"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="21"/>
+      <c r="G16" s="20"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>-4</v>
       </c>
-      <c r="D17" s="19"/>
+      <c r="D17" s="21"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="21"/>
+      <c r="G17" s="20"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>-3</v>
       </c>
-      <c r="D18" s="19"/>
+      <c r="D18" s="21"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1170,7 +1191,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="20"/>
+      <c r="G19" s="19"/>
     </row>
     <row r="20" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20">
@@ -1185,13 +1206,13 @@
       <c r="F20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G20" s="20"/>
+      <c r="G20" s="19"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>0</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="21">
         <v>0</v>
       </c>
       <c r="C21">
@@ -1200,13 +1221,13 @@
       <c r="D21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G21" s="20" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1214,35 +1235,35 @@
       <c r="A22">
         <v>1</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="21"/>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" s="14"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="20"/>
     </row>
     <row r="23" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2</v>
       </c>
-      <c r="B23" s="19"/>
+      <c r="B23" s="21"/>
       <c r="C23">
         <v>2</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="20"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>3</v>
       </c>
-      <c r="B24" s="19"/>
+      <c r="B24" s="21"/>
       <c r="C24">
         <v>3</v>
       </c>
@@ -1253,7 +1274,7 @@
       <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1261,7 +1282,7 @@
       <c r="A25">
         <v>4</v>
       </c>
-      <c r="B25" s="19"/>
+      <c r="B25" s="21"/>
       <c r="C25">
         <v>4</v>
       </c>
@@ -1272,13 +1293,13 @@
       <c r="F25" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="20"/>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>5</v>
       </c>
-      <c r="B26" s="19"/>
+      <c r="B26" s="21"/>
       <c r="C26">
         <v>5</v>
       </c>
@@ -1287,13 +1308,13 @@
         <v>12</v>
       </c>
       <c r="F26" s="22"/>
-      <c r="G26" s="20"/>
+      <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>6</v>
       </c>
-      <c r="B27" s="19"/>
+      <c r="B27" s="21"/>
       <c r="C27">
         <v>6</v>
       </c>
@@ -1304,18 +1325,18 @@
       <c r="F27" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="21" t="s">
+      <c r="G27" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>7</v>
       </c>
-      <c r="B28" s="19"/>
+      <c r="B28" s="21"/>
       <c r="C28">
         <v>7</v>
       </c>
@@ -1324,26 +1345,26 @@
         <v>13</v>
       </c>
       <c r="F28" s="6"/>
-      <c r="G28" s="21"/>
+      <c r="G28" s="20"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>8</v>
       </c>
-      <c r="B29" s="19"/>
+      <c r="B29" s="21"/>
       <c r="C29">
         <v>8</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="12"/>
       <c r="F29" s="6"/>
-      <c r="G29" s="21"/>
+      <c r="G29" s="20"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>9</v>
       </c>
-      <c r="B30" s="19"/>
+      <c r="B30" s="21"/>
       <c r="C30">
         <v>9</v>
       </c>
@@ -1354,7 +1375,7 @@
       <c r="F30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1362,7 +1383,7 @@
       <c r="A31">
         <v>10</v>
       </c>
-      <c r="B31" s="19"/>
+      <c r="B31" s="21"/>
       <c r="C31">
         <v>10</v>
       </c>
@@ -1371,13 +1392,13 @@
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="8"/>
-      <c r="G31" s="20"/>
+      <c r="G31" s="19"/>
     </row>
     <row r="32" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>11</v>
       </c>
-      <c r="B32" s="19"/>
+      <c r="B32" s="21"/>
       <c r="C32">
         <v>11</v>
       </c>
@@ -1386,13 +1407,13 @@
         <v>15</v>
       </c>
       <c r="F32" s="8"/>
-      <c r="G32" s="20"/>
+      <c r="G32" s="19"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>12</v>
       </c>
-      <c r="B33" s="19">
+      <c r="B33" s="21">
         <v>1</v>
       </c>
       <c r="C33">
@@ -1405,18 +1426,18 @@
       <c r="F33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H33" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>13</v>
       </c>
-      <c r="B34" s="19"/>
+      <c r="B34" s="21"/>
       <c r="C34">
         <v>1</v>
       </c>
@@ -1425,13 +1446,13 @@
         <v>16</v>
       </c>
       <c r="F34" s="6"/>
-      <c r="G34" s="21"/>
+      <c r="G34" s="20"/>
     </row>
     <row r="35" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>14</v>
       </c>
-      <c r="B35" s="19"/>
+      <c r="B35" s="21"/>
       <c r="C35">
         <v>2</v>
       </c>
@@ -1440,13 +1461,13 @@
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="21"/>
+      <c r="G35" s="20"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>15</v>
       </c>
-      <c r="B36" s="19"/>
+      <c r="B36" s="21"/>
       <c r="C36">
         <v>3</v>
       </c>
@@ -1457,7 +1478,7 @@
       <c r="F36" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1465,7 +1486,7 @@
       <c r="A37">
         <v>16</v>
       </c>
-      <c r="B37" s="19"/>
+      <c r="B37" s="21"/>
       <c r="C37">
         <v>4</v>
       </c>
@@ -1474,13 +1495,13 @@
       </c>
       <c r="E37" s="11"/>
       <c r="F37" s="8"/>
-      <c r="G37" s="20"/>
+      <c r="G37" s="19"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>17</v>
       </c>
-      <c r="B38" s="19"/>
+      <c r="B38" s="21"/>
       <c r="C38">
         <v>5</v>
       </c>
@@ -1489,13 +1510,13 @@
         <v>12</v>
       </c>
       <c r="F38" s="9"/>
-      <c r="G38" s="20"/>
+      <c r="G38" s="19"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>18</v>
       </c>
-      <c r="B39" s="19"/>
+      <c r="B39" s="21"/>
       <c r="C39">
         <v>6</v>
       </c>
@@ -1506,18 +1527,18 @@
       <c r="F39" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="21" t="s">
+      <c r="G39" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H39" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>19</v>
       </c>
-      <c r="B40" s="19"/>
+      <c r="B40" s="21"/>
       <c r="C40">
         <v>7</v>
       </c>
@@ -1526,26 +1547,26 @@
         <v>13</v>
       </c>
       <c r="F40" s="6"/>
-      <c r="G40" s="21"/>
+      <c r="G40" s="20"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>20</v>
       </c>
-      <c r="B41" s="19"/>
+      <c r="B41" s="21"/>
       <c r="C41">
         <v>8</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="12"/>
       <c r="F41" s="6"/>
-      <c r="G41" s="21"/>
+      <c r="G41" s="20"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>21</v>
       </c>
-      <c r="B42" s="19"/>
+      <c r="B42" s="21"/>
       <c r="C42">
         <v>9</v>
       </c>
@@ -1556,7 +1577,7 @@
       <c r="F42" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="20" t="s">
+      <c r="G42" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1564,7 +1585,7 @@
       <c r="A43">
         <v>22</v>
       </c>
-      <c r="B43" s="19"/>
+      <c r="B43" s="21"/>
       <c r="C43">
         <v>10</v>
       </c>
@@ -1573,13 +1594,13 @@
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="8"/>
-      <c r="G43" s="20"/>
+      <c r="G43" s="19"/>
     </row>
     <row r="44" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>23</v>
       </c>
-      <c r="B44" s="19"/>
+      <c r="B44" s="21"/>
       <c r="C44">
         <v>11</v>
       </c>
@@ -1588,43 +1609,43 @@
         <v>15</v>
       </c>
       <c r="F44" s="8"/>
-      <c r="G44" s="20"/>
+      <c r="G44" s="19"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A45" s="19" t="s">
+      <c r="A45" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
     </row>
     <row r="47" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="19"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
+      <c r="A47" s="21"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A48">
-        <v>45552</v>
-      </c>
-      <c r="B48" s="19">
-        <v>3796</v>
+        <v>45600</v>
+      </c>
+      <c r="B48" s="21">
+        <v>3800</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -1636,18 +1657,18 @@
       <c r="F48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G48" s="21" t="s">
+      <c r="G48" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H48" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A49">
-        <v>45553</v>
-      </c>
-      <c r="B49" s="19"/>
+        <v>45601</v>
+      </c>
+      <c r="B49" s="21"/>
       <c r="C49">
         <v>1</v>
       </c>
@@ -1656,13 +1677,13 @@
         <v>16</v>
       </c>
       <c r="F49" s="6"/>
-      <c r="G49" s="21"/>
+      <c r="G49" s="20"/>
     </row>
     <row r="50" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A50">
-        <v>45554</v>
-      </c>
-      <c r="B50" s="19"/>
+        <v>45602</v>
+      </c>
+      <c r="B50" s="21"/>
       <c r="C50">
         <v>2</v>
       </c>
@@ -1671,13 +1692,13 @@
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="6"/>
-      <c r="G50" s="21"/>
+      <c r="G50" s="20"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51">
-        <v>45555</v>
-      </c>
-      <c r="B51" s="19"/>
+        <v>45603</v>
+      </c>
+      <c r="B51" s="21"/>
       <c r="C51">
         <v>3</v>
       </c>
@@ -1688,15 +1709,15 @@
       <c r="F51" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G51" s="20" t="s">
+      <c r="G51" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A52">
-        <v>45556</v>
-      </c>
-      <c r="B52" s="19"/>
+        <v>45604</v>
+      </c>
+      <c r="B52" s="21"/>
       <c r="C52">
         <v>4</v>
       </c>
@@ -1705,13 +1726,13 @@
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="8"/>
-      <c r="G52" s="20"/>
+      <c r="G52" s="19"/>
     </row>
     <row r="53" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A53">
-        <v>45557</v>
-      </c>
-      <c r="B53" s="19"/>
+        <v>45605</v>
+      </c>
+      <c r="B53" s="21"/>
       <c r="C53">
         <v>5</v>
       </c>
@@ -1720,13 +1741,13 @@
         <v>12</v>
       </c>
       <c r="F53" s="9"/>
-      <c r="G53" s="20"/>
+      <c r="G53" s="19"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A54">
-        <v>45558</v>
-      </c>
-      <c r="B54" s="19"/>
+        <v>45606</v>
+      </c>
+      <c r="B54" s="21"/>
       <c r="C54">
         <v>6</v>
       </c>
@@ -1737,18 +1758,18 @@
       <c r="F54" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G54" s="21" t="s">
+      <c r="G54" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H54" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A55">
-        <v>45559</v>
-      </c>
-      <c r="B55" s="19"/>
+        <v>45607</v>
+      </c>
+      <c r="B55" s="21"/>
       <c r="C55">
         <v>7</v>
       </c>
@@ -1757,26 +1778,26 @@
         <v>13</v>
       </c>
       <c r="F55" s="6"/>
-      <c r="G55" s="21"/>
+      <c r="G55" s="20"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A56">
-        <v>45560</v>
-      </c>
-      <c r="B56" s="19"/>
+        <v>45608</v>
+      </c>
+      <c r="B56" s="21"/>
       <c r="C56">
         <v>8</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="12"/>
       <c r="F56" s="6"/>
-      <c r="G56" s="21"/>
+      <c r="G56" s="20"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A57">
-        <v>45561</v>
-      </c>
-      <c r="B57" s="19"/>
+        <v>45609</v>
+      </c>
+      <c r="B57" s="21"/>
       <c r="C57">
         <v>9</v>
       </c>
@@ -1787,15 +1808,15 @@
       <c r="F57" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G57" s="20" t="s">
+      <c r="G57" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A58">
-        <v>45562</v>
-      </c>
-      <c r="B58" s="19"/>
+        <v>45610</v>
+      </c>
+      <c r="B58" s="21"/>
       <c r="C58">
         <v>10</v>
       </c>
@@ -1804,13 +1825,13 @@
       </c>
       <c r="E58" s="4"/>
       <c r="F58" s="8"/>
-      <c r="G58" s="20"/>
+      <c r="G58" s="19"/>
     </row>
     <row r="59" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A59">
-        <v>45563</v>
-      </c>
-      <c r="B59" s="19"/>
+        <v>45611</v>
+      </c>
+      <c r="B59" s="21"/>
       <c r="C59">
         <v>11</v>
       </c>
@@ -1819,11 +1840,11 @@
         <v>15</v>
       </c>
       <c r="F59" s="8"/>
-      <c r="G59" s="20"/>
+      <c r="G59" s="19"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A60">
-        <v>45564</v>
+        <v>45612</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>21</v>
@@ -1832,304 +1853,304 @@
       <c r="F60" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G60" s="21" t="s">
+      <c r="G60" s="20" t="s">
         <v>5</v>
       </c>
       <c r="H60" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A61">
-        <v>45565</v>
+        <v>45613</v>
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F61" s="6"/>
-      <c r="G61" s="21"/>
+      <c r="G61" s="20"/>
     </row>
     <row r="62" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A62">
-        <v>45566</v>
+        <v>45614</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="6"/>
-      <c r="G62" s="21"/>
+      <c r="G62" s="20"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A63">
-        <v>45567</v>
+        <v>45615</v>
       </c>
       <c r="D63" s="1"/>
       <c r="F63" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G63" s="20" t="s">
+      <c r="G63" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A64">
-        <v>45568</v>
+        <v>45616</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F64" s="8"/>
-      <c r="G64" s="20"/>
+      <c r="G64" s="19"/>
     </row>
     <row r="65" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A65">
-        <v>45569</v>
-      </c>
-      <c r="D65" s="19" t="s">
+        <v>45617</v>
+      </c>
+      <c r="D65" s="21" t="s">
         <v>22</v>
       </c>
       <c r="F65" s="9"/>
-      <c r="G65" s="20"/>
+      <c r="G65" s="19"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66">
-        <v>45570</v>
-      </c>
-      <c r="D66" s="19"/>
-      <c r="G66" s="21" t="s">
+        <v>45618</v>
+      </c>
+      <c r="D66" s="21"/>
+      <c r="G66" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A67">
-        <v>45571</v>
-      </c>
-      <c r="D67" s="19"/>
-      <c r="G67" s="21"/>
+        <v>45619</v>
+      </c>
+      <c r="D67" s="21"/>
+      <c r="G67" s="20"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68">
-        <v>45572</v>
-      </c>
-      <c r="D68" s="19"/>
-      <c r="G68" s="21"/>
+        <v>45620</v>
+      </c>
+      <c r="D68" s="21"/>
+      <c r="G68" s="20"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69">
-        <v>45573</v>
-      </c>
-      <c r="D69" s="19"/>
-      <c r="G69" s="20" t="s">
+        <v>45621</v>
+      </c>
+      <c r="D69" s="21"/>
+      <c r="G69" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A70">
-        <v>45574</v>
-      </c>
-      <c r="D70" s="19"/>
-      <c r="G70" s="20"/>
+        <v>45622</v>
+      </c>
+      <c r="D70" s="21"/>
+      <c r="G70" s="19"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71">
-        <v>45575</v>
-      </c>
-      <c r="D71" s="19"/>
-      <c r="G71" s="20"/>
+        <v>45623</v>
+      </c>
+      <c r="D71" s="21"/>
+      <c r="G71" s="19"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72">
-        <v>45576</v>
-      </c>
-      <c r="D72" s="19"/>
-      <c r="G72" s="21" t="s">
+        <v>45624</v>
+      </c>
+      <c r="D72" s="21"/>
+      <c r="G72" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A73">
-        <v>45577</v>
-      </c>
-      <c r="D73" s="19"/>
-      <c r="G73" s="21"/>
+        <v>45625</v>
+      </c>
+      <c r="D73" s="21"/>
+      <c r="G73" s="20"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74">
-        <v>45578</v>
-      </c>
-      <c r="D74" s="19"/>
-      <c r="G74" s="21"/>
+        <v>45626</v>
+      </c>
+      <c r="D74" s="21"/>
+      <c r="G74" s="20"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75">
-        <v>45579</v>
-      </c>
-      <c r="D75" s="19"/>
-      <c r="G75" s="20" t="s">
+        <v>45627</v>
+      </c>
+      <c r="D75" s="21"/>
+      <c r="G75" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A76">
-        <v>45580</v>
-      </c>
-      <c r="D76" s="19"/>
-      <c r="G76" s="20"/>
+        <v>45628</v>
+      </c>
+      <c r="D76" s="21"/>
+      <c r="G76" s="19"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77">
-        <v>45581</v>
-      </c>
-      <c r="D77" s="19"/>
-      <c r="G77" s="20"/>
+        <v>45629</v>
+      </c>
+      <c r="D77" s="21"/>
+      <c r="G77" s="19"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78">
-        <v>45582</v>
-      </c>
-      <c r="D78" s="19"/>
-      <c r="G78" s="21" t="s">
+        <v>45630</v>
+      </c>
+      <c r="D78" s="21"/>
+      <c r="G78" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A79">
-        <v>45583</v>
-      </c>
-      <c r="D79" s="19"/>
-      <c r="G79" s="21"/>
+        <v>45631</v>
+      </c>
+      <c r="D79" s="21"/>
+      <c r="G79" s="20"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80">
-        <v>45584</v>
+        <v>45632</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G80" s="21"/>
+      <c r="G80" s="20"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81">
-        <v>45585</v>
-      </c>
-      <c r="D81" s="19" t="s">
+        <v>45633</v>
+      </c>
+      <c r="D81" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G81" s="20" t="s">
+      <c r="G81" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A82">
-        <v>45586</v>
-      </c>
-      <c r="D82" s="19"/>
-      <c r="G82" s="20"/>
+        <v>45634</v>
+      </c>
+      <c r="D82" s="21"/>
+      <c r="G82" s="19"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83">
-        <v>45587</v>
-      </c>
-      <c r="D83" s="19"/>
-      <c r="G83" s="20"/>
+        <v>45635</v>
+      </c>
+      <c r="D83" s="21"/>
+      <c r="G83" s="19"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84">
-        <v>45588</v>
-      </c>
-      <c r="D84" s="19"/>
-      <c r="G84" s="21" t="s">
+        <v>45636</v>
+      </c>
+      <c r="D84" s="21"/>
+      <c r="G84" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A85">
-        <v>45589</v>
-      </c>
-      <c r="D85" s="19"/>
-      <c r="G85" s="21"/>
+        <v>45637</v>
+      </c>
+      <c r="D85" s="21"/>
+      <c r="G85" s="20"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86">
-        <v>45590</v>
-      </c>
-      <c r="D86" s="19"/>
-      <c r="G86" s="21"/>
+        <v>45638</v>
+      </c>
+      <c r="D86" s="21"/>
+      <c r="G86" s="20"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87">
-        <v>45591</v>
-      </c>
-      <c r="D87" s="19"/>
-      <c r="G87" s="20" t="s">
+        <v>45639</v>
+      </c>
+      <c r="D87" s="21"/>
+      <c r="G87" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A88">
-        <v>45592</v>
-      </c>
-      <c r="D88" s="19"/>
-      <c r="G88" s="20"/>
+        <v>45640</v>
+      </c>
+      <c r="D88" s="21"/>
+      <c r="G88" s="19"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89">
-        <v>45593</v>
-      </c>
-      <c r="D89" s="19"/>
-      <c r="G89" s="20"/>
+        <v>45641</v>
+      </c>
+      <c r="D89" s="21"/>
+      <c r="G89" s="19"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90">
-        <v>45594</v>
-      </c>
-      <c r="D90" s="19"/>
-      <c r="G90" s="21" t="s">
+        <v>45642</v>
+      </c>
+      <c r="D90" s="21"/>
+      <c r="G90" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A91">
-        <v>45595</v>
-      </c>
-      <c r="D91" s="19"/>
-      <c r="G91" s="21"/>
+        <v>45643</v>
+      </c>
+      <c r="D91" s="21"/>
+      <c r="G91" s="20"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92">
-        <v>45596</v>
-      </c>
-      <c r="D92" s="19"/>
-      <c r="G92" s="21"/>
+        <v>45644</v>
+      </c>
+      <c r="D92" s="21"/>
+      <c r="G92" s="20"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93">
-        <v>45597</v>
-      </c>
-      <c r="D93" s="19"/>
-      <c r="G93" s="20" t="s">
+        <v>45645</v>
+      </c>
+      <c r="D93" s="21"/>
+      <c r="G93" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A94">
-        <v>45598</v>
-      </c>
-      <c r="D94" s="19"/>
-      <c r="G94" s="20"/>
+        <v>45646</v>
+      </c>
+      <c r="D94" s="21"/>
+      <c r="G94" s="19"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95">
-        <v>45599</v>
-      </c>
-      <c r="D95" s="19"/>
-      <c r="G95" s="20"/>
+        <v>45647</v>
+      </c>
+      <c r="D95" s="21"/>
+      <c r="G95" s="19"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96">
-        <v>45600</v>
+        <v>45648</v>
       </c>
       <c r="D96" t="s">
         <v>26</v>
@@ -2142,147 +2163,147 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A98">
-        <v>45744</v>
-      </c>
-      <c r="D98" s="19" t="s">
+        <v>45792</v>
+      </c>
+      <c r="D98" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G98" s="21" t="s">
+      <c r="G98" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A99">
-        <v>45745</v>
-      </c>
-      <c r="D99" s="19"/>
-      <c r="G99" s="21"/>
+        <v>45793</v>
+      </c>
+      <c r="D99" s="21"/>
+      <c r="G99" s="20"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A100">
-        <v>45746</v>
-      </c>
-      <c r="D100" s="19"/>
-      <c r="G100" s="21"/>
+        <v>45794</v>
+      </c>
+      <c r="D100" s="21"/>
+      <c r="G100" s="20"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A101">
-        <v>45747</v>
-      </c>
-      <c r="D101" s="19"/>
-      <c r="G101" s="20" t="s">
+        <v>45795</v>
+      </c>
+      <c r="D101" s="21"/>
+      <c r="G101" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A102">
-        <v>45748</v>
-      </c>
-      <c r="D102" s="19"/>
-      <c r="G102" s="20"/>
+        <v>45796</v>
+      </c>
+      <c r="D102" s="21"/>
+      <c r="G102" s="19"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103">
-        <v>45749</v>
-      </c>
-      <c r="D103" s="19"/>
-      <c r="G103" s="20"/>
+        <v>45797</v>
+      </c>
+      <c r="D103" s="21"/>
+      <c r="G103" s="19"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A104">
-        <v>45750</v>
-      </c>
-      <c r="D104" s="19"/>
-      <c r="G104" s="21" t="s">
+        <v>45798</v>
+      </c>
+      <c r="D104" s="21"/>
+      <c r="G104" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A105">
-        <v>45751</v>
-      </c>
-      <c r="D105" s="19"/>
-      <c r="G105" s="21"/>
+        <v>45799</v>
+      </c>
+      <c r="D105" s="21"/>
+      <c r="G105" s="20"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106">
-        <v>45752</v>
-      </c>
-      <c r="D106" s="19"/>
-      <c r="G106" s="21"/>
+        <v>45800</v>
+      </c>
+      <c r="D106" s="21"/>
+      <c r="G106" s="20"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107">
-        <v>45753</v>
-      </c>
-      <c r="D107" s="19"/>
-      <c r="G107" s="20" t="s">
+        <v>45801</v>
+      </c>
+      <c r="D107" s="21"/>
+      <c r="G107" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A108">
-        <v>45754</v>
-      </c>
-      <c r="D108" s="19"/>
-      <c r="G108" s="20"/>
+        <v>45802</v>
+      </c>
+      <c r="D108" s="21"/>
+      <c r="G108" s="19"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109">
-        <v>45755</v>
-      </c>
-      <c r="D109" s="19"/>
-      <c r="G109" s="20"/>
+        <v>45803</v>
+      </c>
+      <c r="D109" s="21"/>
+      <c r="G109" s="19"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A110">
-        <v>45756</v>
-      </c>
-      <c r="D110" s="19"/>
-      <c r="G110" s="21" t="s">
+        <v>45804</v>
+      </c>
+      <c r="D110" s="21"/>
+      <c r="G110" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A111">
-        <v>45757</v>
-      </c>
-      <c r="D111" s="19"/>
-      <c r="G111" s="21"/>
+        <v>45805</v>
+      </c>
+      <c r="D111" s="21"/>
+      <c r="G111" s="20"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112">
-        <v>45758</v>
-      </c>
-      <c r="D112" s="19"/>
-      <c r="G112" s="21"/>
+        <v>45806</v>
+      </c>
+      <c r="D112" s="21"/>
+      <c r="G112" s="20"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113">
-        <v>45759</v>
+        <v>45807</v>
       </c>
       <c r="D113" t="s">
         <v>28</v>
       </c>
-      <c r="G113" s="20" t="s">
+      <c r="G113" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A114">
-        <v>45760</v>
-      </c>
-      <c r="G114" s="20"/>
+        <v>45808</v>
+      </c>
+      <c r="G114" s="19"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115">
-        <v>45761</v>
-      </c>
-      <c r="G115" s="20"/>
+        <v>45809</v>
+      </c>
+      <c r="G115" s="19"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116">
-        <v>45762</v>
+        <v>45810</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>17</v>
@@ -2294,7 +2315,7 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A117">
-        <v>45763</v>
+        <v>45811</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>4</v>
@@ -2307,9 +2328,9 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A118">
-        <v>45764</v>
-      </c>
-      <c r="D118" s="19" t="s">
+        <v>45812</v>
+      </c>
+      <c r="D118" s="21" t="s">
         <v>31</v>
       </c>
       <c r="E118" s="1"/>
@@ -2318,145 +2339,145 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A119">
-        <v>45765</v>
-      </c>
-      <c r="D119" s="19"/>
+        <v>45813</v>
+      </c>
+      <c r="D119" s="21"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
-      <c r="G119" s="20" t="s">
+      <c r="G119" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A120">
-        <v>45766</v>
-      </c>
-      <c r="D120" s="19"/>
+        <v>45814</v>
+      </c>
+      <c r="D120" s="21"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
-      <c r="G120" s="20"/>
+      <c r="G120" s="19"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121">
-        <v>45767</v>
-      </c>
-      <c r="D121" s="19"/>
+        <v>45815</v>
+      </c>
+      <c r="D121" s="21"/>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
-      <c r="G121" s="20"/>
+      <c r="G121" s="19"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122">
-        <v>45768</v>
-      </c>
-      <c r="D122" s="19"/>
+        <v>45816</v>
+      </c>
+      <c r="D122" s="21"/>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
-      <c r="G122" s="21" t="s">
+      <c r="G122" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A123">
-        <v>45769</v>
-      </c>
-      <c r="D123" s="19"/>
+        <v>45817</v>
+      </c>
+      <c r="D123" s="21"/>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
-      <c r="G123" s="21"/>
+      <c r="G123" s="20"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124">
-        <v>45770</v>
-      </c>
-      <c r="D124" s="19"/>
+        <v>45818</v>
+      </c>
+      <c r="D124" s="21"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="21"/>
+      <c r="G124" s="20"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125">
-        <v>45771</v>
-      </c>
-      <c r="D125" s="19"/>
+        <v>45819</v>
+      </c>
+      <c r="D125" s="21"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
-      <c r="G125" s="20" t="s">
+      <c r="G125" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A126">
-        <v>45772</v>
-      </c>
-      <c r="D126" s="19"/>
+        <v>45820</v>
+      </c>
+      <c r="D126" s="21"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-      <c r="G126" s="20"/>
+      <c r="G126" s="19"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127">
-        <v>45773</v>
-      </c>
-      <c r="D127" s="19"/>
+        <v>45821</v>
+      </c>
+      <c r="D127" s="21"/>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
-      <c r="G127" s="20"/>
+      <c r="G127" s="19"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128">
-        <v>45774</v>
-      </c>
-      <c r="D128" s="19"/>
+        <v>45822</v>
+      </c>
+      <c r="D128" s="21"/>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
-      <c r="G128" s="21" t="s">
+      <c r="G128" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A129">
-        <v>45775</v>
-      </c>
-      <c r="D129" s="19"/>
+        <v>45823</v>
+      </c>
+      <c r="D129" s="21"/>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
-      <c r="G129" s="21"/>
+      <c r="G129" s="20"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130">
-        <v>45776</v>
-      </c>
-      <c r="D130" s="19"/>
+        <v>45824</v>
+      </c>
+      <c r="D130" s="21"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
-      <c r="G130" s="21"/>
+      <c r="G130" s="20"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131">
-        <v>45777</v>
-      </c>
-      <c r="D131" s="19"/>
+        <v>45825</v>
+      </c>
+      <c r="D131" s="21"/>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
-      <c r="G131" s="20" t="s">
+      <c r="G131" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A132">
-        <v>45778</v>
+        <v>45826</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
-      <c r="G132" s="20"/>
+      <c r="G132" s="19"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133">
-        <v>45779</v>
+        <v>45827</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>10</v>
@@ -2467,18 +2488,38 @@
       <c r="F133" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G133" s="20"/>
+      <c r="G133" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="D118:D131"/>
+    <mergeCell ref="D5:D18"/>
+    <mergeCell ref="G107:G109"/>
+    <mergeCell ref="G110:G112"/>
+    <mergeCell ref="G113:G115"/>
+    <mergeCell ref="G119:G121"/>
+    <mergeCell ref="G122:G124"/>
+    <mergeCell ref="G125:G127"/>
+    <mergeCell ref="G128:G130"/>
+    <mergeCell ref="G131:G133"/>
+    <mergeCell ref="D81:D95"/>
+    <mergeCell ref="G72:G74"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="G81:G83"/>
+    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="G93:G95"/>
+    <mergeCell ref="G98:G100"/>
+    <mergeCell ref="D98:D112"/>
+    <mergeCell ref="G101:G103"/>
+    <mergeCell ref="G104:G106"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="D65:D79"/>
     <mergeCell ref="B21:B32"/>
     <mergeCell ref="B33:B44"/>
     <mergeCell ref="A45:G47"/>
@@ -2495,34 +2536,14 @@
     <mergeCell ref="E21:E23"/>
     <mergeCell ref="G33:G35"/>
     <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="D65:D79"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="G93:G95"/>
-    <mergeCell ref="G98:G100"/>
-    <mergeCell ref="D98:D112"/>
-    <mergeCell ref="G101:G103"/>
-    <mergeCell ref="G104:G106"/>
-    <mergeCell ref="D118:D131"/>
-    <mergeCell ref="D5:D18"/>
-    <mergeCell ref="G107:G109"/>
-    <mergeCell ref="G110:G112"/>
-    <mergeCell ref="G113:G115"/>
-    <mergeCell ref="G119:G121"/>
-    <mergeCell ref="G122:G124"/>
-    <mergeCell ref="G125:G127"/>
-    <mergeCell ref="G128:G130"/>
-    <mergeCell ref="G131:G133"/>
-    <mergeCell ref="D81:D95"/>
-    <mergeCell ref="G72:G74"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="G78:G80"/>
-    <mergeCell ref="G81:G83"/>
-    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update SM1 timing sequence for stability
</commit_message>
<xml_diff>
--- a/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
+++ b/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3FC44E-CB62-42CC-853C-55730C589838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ECC6378-3472-4726-82C1-1DDB88886B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="18676" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -457,7 +457,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -515,16 +515,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -853,8 +856,7 @@
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="4" max="4" width="14.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14.46484375" customWidth="1"/>
-    <col min="6" max="6" width="12.86328125" customWidth="1"/>
+    <col min="5" max="6" width="14.46484375" customWidth="1"/>
     <col min="7" max="7" width="12.59765625" customWidth="1"/>
     <col min="10" max="10" width="13.06640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.1328125" bestFit="1" customWidth="1"/>
@@ -931,7 +933,7 @@
       <c r="A5">
         <v>-16</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="1"/>
@@ -942,10 +944,10 @@
       <c r="A6">
         <v>-15</v>
       </c>
-      <c r="D6" s="21"/>
+      <c r="D6" s="19"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -953,10 +955,10 @@
       <c r="A7">
         <v>-14</v>
       </c>
-      <c r="D7" s="21"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="19"/>
+      <c r="G7" s="20"/>
       <c r="J7" t="s">
         <v>51</v>
       </c>
@@ -977,10 +979,10 @@
       <c r="A8">
         <v>-13</v>
       </c>
-      <c r="D8" s="21"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="19"/>
+      <c r="G8" s="20"/>
       <c r="J8" s="17">
         <v>0</v>
       </c>
@@ -998,10 +1000,10 @@
       <c r="A9">
         <v>-12</v>
       </c>
-      <c r="D9" s="21"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="21" t="s">
         <v>5</v>
       </c>
       <c r="J9">
@@ -1024,10 +1026,10 @@
       <c r="A10">
         <v>-11</v>
       </c>
-      <c r="D10" s="21"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="20"/>
+      <c r="G10" s="21"/>
       <c r="J10">
         <v>359</v>
       </c>
@@ -1048,10 +1050,10 @@
       <c r="A11">
         <v>-10</v>
       </c>
-      <c r="D11" s="21"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="20"/>
+      <c r="G11" s="21"/>
       <c r="J11">
         <v>1400</v>
       </c>
@@ -1072,10 +1074,10 @@
       <c r="A12">
         <v>-9</v>
       </c>
-      <c r="D12" s="21"/>
+      <c r="D12" s="19"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="20" t="s">
         <v>6</v>
       </c>
       <c r="J12">
@@ -1098,10 +1100,10 @@
       <c r="A13">
         <v>-8</v>
       </c>
-      <c r="D13" s="21"/>
+      <c r="D13" s="19"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="19"/>
+      <c r="G13" s="20"/>
       <c r="J13">
         <v>4525</v>
       </c>
@@ -1122,10 +1124,10 @@
       <c r="A14">
         <v>-7</v>
       </c>
-      <c r="D14" s="21"/>
+      <c r="D14" s="19"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="19"/>
+      <c r="G14" s="20"/>
       <c r="J14">
         <v>6609</v>
       </c>
@@ -1146,10 +1148,10 @@
       <c r="A15">
         <v>-6</v>
       </c>
-      <c r="D15" s="21"/>
+      <c r="D15" s="19"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1157,28 +1159,28 @@
       <c r="A16">
         <v>-5</v>
       </c>
-      <c r="D16" s="21"/>
+      <c r="D16" s="19"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="20"/>
+      <c r="G16" s="21"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>-4</v>
       </c>
-      <c r="D17" s="21"/>
+      <c r="D17" s="19"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="20"/>
+      <c r="G17" s="21"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>-3</v>
       </c>
-      <c r="D18" s="21"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1191,7 +1193,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="19"/>
+      <c r="G19" s="20"/>
     </row>
     <row r="20" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20">
@@ -1206,13 +1208,13 @@
       <c r="F20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G20" s="19"/>
+      <c r="G20" s="20"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>0</v>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="19">
         <v>0</v>
       </c>
       <c r="C21">
@@ -1221,60 +1223,60 @@
       <c r="D21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="21" t="s">
+      <c r="E21" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>1</v>
       </c>
-      <c r="B22" s="21"/>
+      <c r="B22" s="19"/>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" s="14"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="20"/>
-    </row>
-    <row r="23" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="E22" s="22"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="21"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>2</v>
       </c>
-      <c r="B23" s="21"/>
+      <c r="B23" s="19"/>
       <c r="C23">
         <v>2</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="20"/>
+      <c r="E23" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="19"/>
+      <c r="G23" s="21"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>3</v>
       </c>
-      <c r="B24" s="21"/>
+      <c r="B24" s="19"/>
       <c r="C24">
         <v>3</v>
       </c>
       <c r="D24" s="15"/>
-      <c r="E24" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="E24" s="11"/>
       <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1282,50 +1284,52 @@
       <c r="A25">
         <v>4</v>
       </c>
-      <c r="B25" s="21"/>
+      <c r="B25" s="19"/>
       <c r="C25">
         <v>4</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="11"/>
+      <c r="E25" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="F25" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="19"/>
+      <c r="G25" s="20"/>
     </row>
     <row r="26" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>5</v>
       </c>
-      <c r="B26" s="21"/>
+      <c r="B26" s="19"/>
       <c r="C26">
         <v>5</v>
       </c>
       <c r="D26" s="15"/>
-      <c r="E26" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="22"/>
-      <c r="G26" s="19"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="20"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>6</v>
       </c>
-      <c r="B27" s="21"/>
+      <c r="B27" s="19"/>
       <c r="C27">
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="11"/>
+      <c r="E27" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="F27" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H27" t="s">
@@ -1336,46 +1340,44 @@
       <c r="A28">
         <v>7</v>
       </c>
-      <c r="B28" s="21"/>
+      <c r="B28" s="19"/>
       <c r="C28">
         <v>7</v>
       </c>
       <c r="D28" s="2"/>
-      <c r="E28" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="E28" s="12"/>
       <c r="F28" s="6"/>
-      <c r="G28" s="20"/>
+      <c r="G28" s="21"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>8</v>
       </c>
-      <c r="B29" s="21"/>
+      <c r="B29" s="19"/>
       <c r="C29">
         <v>8</v>
       </c>
       <c r="D29" s="2"/>
-      <c r="E29" s="12"/>
+      <c r="E29" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="F29" s="6"/>
-      <c r="G29" s="20"/>
+      <c r="G29" s="21"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>9</v>
       </c>
-      <c r="B30" s="21"/>
+      <c r="B30" s="19"/>
       <c r="C30">
         <v>9</v>
       </c>
       <c r="D30" s="2"/>
-      <c r="E30" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="E30" s="4"/>
       <c r="F30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="19" t="s">
+      <c r="G30" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1383,37 +1385,37 @@
       <c r="A31">
         <v>10</v>
       </c>
-      <c r="B31" s="21"/>
+      <c r="B31" s="19"/>
       <c r="C31">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F31" s="8"/>
-      <c r="G31" s="19"/>
+      <c r="G31" s="20"/>
     </row>
     <row r="32" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>11</v>
       </c>
-      <c r="B32" s="21"/>
+      <c r="B32" s="19"/>
       <c r="C32">
         <v>11</v>
       </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E32" s="4"/>
       <c r="F32" s="8"/>
-      <c r="G32" s="19"/>
+      <c r="G32" s="20"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>12</v>
       </c>
-      <c r="B33" s="21">
+      <c r="B33" s="19">
         <v>1</v>
       </c>
       <c r="C33">
@@ -1422,63 +1424,63 @@
       <c r="D33" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="4"/>
+      <c r="E33" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="F33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H33" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>13</v>
       </c>
-      <c r="B34" s="21"/>
+      <c r="B34" s="19"/>
       <c r="C34">
         <v>1</v>
       </c>
       <c r="D34" s="14"/>
-      <c r="E34" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="E34" s="5"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="20"/>
-    </row>
-    <row r="35" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G34" s="21"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>14</v>
       </c>
-      <c r="B35" s="21"/>
+      <c r="B35" s="19"/>
       <c r="C35">
         <v>2</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="5"/>
+      <c r="E35" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="F35" s="6"/>
-      <c r="G35" s="20"/>
+      <c r="G35" s="21"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>15</v>
       </c>
-      <c r="B36" s="21"/>
+      <c r="B36" s="19"/>
       <c r="C36">
         <v>3</v>
       </c>
       <c r="D36" s="15"/>
-      <c r="E36" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="E36" s="11"/>
       <c r="F36" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="19" t="s">
+      <c r="G36" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1486,48 +1488,50 @@
       <c r="A37">
         <v>16</v>
       </c>
-      <c r="B37" s="21"/>
+      <c r="B37" s="19"/>
       <c r="C37">
         <v>4</v>
       </c>
       <c r="D37" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E37" s="11"/>
+      <c r="E37" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="F37" s="8"/>
-      <c r="G37" s="19"/>
+      <c r="G37" s="20"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>17</v>
       </c>
-      <c r="B38" s="21"/>
+      <c r="B38" s="19"/>
       <c r="C38">
         <v>5</v>
       </c>
       <c r="D38" s="15"/>
-      <c r="E38" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="E38" s="12"/>
       <c r="F38" s="9"/>
-      <c r="G38" s="19"/>
+      <c r="G38" s="20"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>18</v>
       </c>
-      <c r="B39" s="21"/>
+      <c r="B39" s="19"/>
       <c r="C39">
         <v>6</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="11"/>
+      <c r="E39" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="F39" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="G39" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H39" t="s">
@@ -1538,46 +1542,44 @@
       <c r="A40">
         <v>19</v>
       </c>
-      <c r="B40" s="21"/>
+      <c r="B40" s="19"/>
       <c r="C40">
         <v>7</v>
       </c>
       <c r="D40" s="2"/>
-      <c r="E40" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="E40" s="12"/>
       <c r="F40" s="6"/>
-      <c r="G40" s="20"/>
+      <c r="G40" s="21"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>20</v>
       </c>
-      <c r="B41" s="21"/>
+      <c r="B41" s="19"/>
       <c r="C41">
         <v>8</v>
       </c>
       <c r="D41" s="2"/>
-      <c r="E41" s="12"/>
+      <c r="E41" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="F41" s="6"/>
-      <c r="G41" s="20"/>
+      <c r="G41" s="21"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>21</v>
       </c>
-      <c r="B42" s="21"/>
+      <c r="B42" s="19"/>
       <c r="C42">
         <v>9</v>
       </c>
       <c r="D42" s="2"/>
-      <c r="E42" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="E42" s="4"/>
       <c r="F42" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="19" t="s">
+      <c r="G42" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1585,66 +1587,66 @@
       <c r="A43">
         <v>22</v>
       </c>
-      <c r="B43" s="21"/>
+      <c r="B43" s="19"/>
       <c r="C43">
         <v>10</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="19"/>
+      <c r="G43" s="20"/>
     </row>
     <row r="44" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>23</v>
       </c>
-      <c r="B44" s="21"/>
+      <c r="B44" s="19"/>
       <c r="C44">
         <v>11</v>
       </c>
       <c r="D44" s="3"/>
-      <c r="E44" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E44" s="4"/>
       <c r="F44" s="8"/>
-      <c r="G44" s="19"/>
+      <c r="G44" s="20"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
-      <c r="G45" s="21"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="19"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A46" s="21"/>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
+      <c r="A46" s="19"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="19"/>
     </row>
     <row r="47" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="21"/>
-      <c r="B47" s="21"/>
-      <c r="C47" s="21"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="21"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="21"/>
+      <c r="A47" s="19"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>45600</v>
       </c>
-      <c r="B48" s="21">
+      <c r="B48" s="19">
         <v>3800</v>
       </c>
       <c r="C48">
@@ -1653,63 +1655,63 @@
       <c r="D48" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E48" s="4"/>
+      <c r="E48" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="F48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G48" s="20" t="s">
+      <c r="G48" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H48" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>45601</v>
       </c>
-      <c r="B49" s="21"/>
+      <c r="B49" s="19"/>
       <c r="C49">
         <v>1</v>
       </c>
       <c r="D49" s="14"/>
-      <c r="E49" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="E49" s="5"/>
       <c r="F49" s="6"/>
-      <c r="G49" s="20"/>
-    </row>
-    <row r="50" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G49" s="21"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>45602</v>
       </c>
-      <c r="B50" s="21"/>
+      <c r="B50" s="19"/>
       <c r="C50">
         <v>2</v>
       </c>
       <c r="D50" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E50" s="5"/>
+      <c r="E50" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="F50" s="6"/>
-      <c r="G50" s="20"/>
+      <c r="G50" s="21"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>45603</v>
       </c>
-      <c r="B51" s="21"/>
+      <c r="B51" s="19"/>
       <c r="C51">
         <v>3</v>
       </c>
       <c r="D51" s="15"/>
-      <c r="E51" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="E51" s="11"/>
       <c r="F51" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G51" s="19" t="s">
+      <c r="G51" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1717,48 +1719,50 @@
       <c r="A52">
         <v>45604</v>
       </c>
-      <c r="B52" s="21"/>
+      <c r="B52" s="19"/>
       <c r="C52">
         <v>4</v>
       </c>
       <c r="D52" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E52" s="11"/>
+      <c r="E52" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="F52" s="8"/>
-      <c r="G52" s="19"/>
+      <c r="G52" s="20"/>
     </row>
     <row r="53" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>45605</v>
       </c>
-      <c r="B53" s="21"/>
+      <c r="B53" s="19"/>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53" s="15"/>
-      <c r="E53" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="E53" s="12"/>
       <c r="F53" s="9"/>
-      <c r="G53" s="19"/>
+      <c r="G53" s="20"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>45606</v>
       </c>
-      <c r="B54" s="21"/>
+      <c r="B54" s="19"/>
       <c r="C54">
         <v>6</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E54" s="11"/>
+      <c r="E54" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="F54" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G54" s="20" t="s">
+      <c r="G54" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H54" t="s">
@@ -1769,46 +1773,44 @@
       <c r="A55">
         <v>45607</v>
       </c>
-      <c r="B55" s="21"/>
+      <c r="B55" s="19"/>
       <c r="C55">
         <v>7</v>
       </c>
       <c r="D55" s="2"/>
-      <c r="E55" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="E55" s="12"/>
       <c r="F55" s="6"/>
-      <c r="G55" s="20"/>
+      <c r="G55" s="21"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>45608</v>
       </c>
-      <c r="B56" s="21"/>
+      <c r="B56" s="19"/>
       <c r="C56">
         <v>8</v>
       </c>
       <c r="D56" s="2"/>
-      <c r="E56" s="12"/>
+      <c r="E56" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="F56" s="6"/>
-      <c r="G56" s="20"/>
+      <c r="G56" s="21"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>45609</v>
       </c>
-      <c r="B57" s="21"/>
+      <c r="B57" s="19"/>
       <c r="C57">
         <v>9</v>
       </c>
       <c r="D57" s="2"/>
-      <c r="E57" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="E57" s="4"/>
       <c r="F57" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G57" s="19" t="s">
+      <c r="G57" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1816,31 +1818,31 @@
       <c r="A58">
         <v>45610</v>
       </c>
-      <c r="B58" s="21"/>
+      <c r="B58" s="19"/>
       <c r="C58">
         <v>10</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E58" s="4"/>
+      <c r="E58" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F58" s="8"/>
-      <c r="G58" s="19"/>
+      <c r="G58" s="20"/>
     </row>
     <row r="59" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>45611</v>
       </c>
-      <c r="B59" s="21"/>
+      <c r="B59" s="19"/>
       <c r="C59">
         <v>11</v>
       </c>
       <c r="D59" s="3"/>
-      <c r="E59" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E59" s="4"/>
       <c r="F59" s="8"/>
-      <c r="G59" s="19"/>
+      <c r="G59" s="20"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A60">
@@ -1849,38 +1851,37 @@
       <c r="D60" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E60" s="4"/>
+      <c r="E60" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="F60" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G60" s="20" t="s">
+      <c r="G60" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H60" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>45613</v>
       </c>
       <c r="D61" s="1"/>
-      <c r="E61" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="E61" s="5"/>
       <c r="F61" s="6"/>
-      <c r="G61" s="20"/>
-    </row>
-    <row r="62" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G61" s="21"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>45614</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E62" s="5"/>
       <c r="F62" s="6"/>
-      <c r="G62" s="20"/>
+      <c r="G62" s="21"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A63">
@@ -1890,7 +1891,7 @@
       <c r="F63" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G63" s="19" t="s">
+      <c r="G63" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1902,24 +1903,24 @@
         <v>21</v>
       </c>
       <c r="F64" s="8"/>
-      <c r="G64" s="19"/>
+      <c r="G64" s="20"/>
     </row>
     <row r="65" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>45617</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="19" t="s">
         <v>22</v>
       </c>
       <c r="F65" s="9"/>
-      <c r="G65" s="19"/>
+      <c r="G65" s="20"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>45618</v>
       </c>
-      <c r="D66" s="21"/>
-      <c r="G66" s="20" t="s">
+      <c r="D66" s="19"/>
+      <c r="G66" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1927,22 +1928,22 @@
       <c r="A67">
         <v>45619</v>
       </c>
-      <c r="D67" s="21"/>
-      <c r="G67" s="20"/>
+      <c r="D67" s="19"/>
+      <c r="G67" s="21"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>45620</v>
       </c>
-      <c r="D68" s="21"/>
-      <c r="G68" s="20"/>
+      <c r="D68" s="19"/>
+      <c r="G68" s="21"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>45621</v>
       </c>
-      <c r="D69" s="21"/>
-      <c r="G69" s="19" t="s">
+      <c r="D69" s="19"/>
+      <c r="G69" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1950,22 +1951,22 @@
       <c r="A70">
         <v>45622</v>
       </c>
-      <c r="D70" s="21"/>
-      <c r="G70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="G70" s="20"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>45623</v>
       </c>
-      <c r="D71" s="21"/>
-      <c r="G71" s="19"/>
+      <c r="D71" s="19"/>
+      <c r="G71" s="20"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>45624</v>
       </c>
-      <c r="D72" s="21"/>
-      <c r="G72" s="20" t="s">
+      <c r="D72" s="19"/>
+      <c r="G72" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1973,22 +1974,22 @@
       <c r="A73">
         <v>45625</v>
       </c>
-      <c r="D73" s="21"/>
-      <c r="G73" s="20"/>
+      <c r="D73" s="19"/>
+      <c r="G73" s="21"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>45626</v>
       </c>
-      <c r="D74" s="21"/>
-      <c r="G74" s="20"/>
+      <c r="D74" s="19"/>
+      <c r="G74" s="21"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>45627</v>
       </c>
-      <c r="D75" s="21"/>
-      <c r="G75" s="19" t="s">
+      <c r="D75" s="19"/>
+      <c r="G75" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1996,22 +1997,22 @@
       <c r="A76">
         <v>45628</v>
       </c>
-      <c r="D76" s="21"/>
-      <c r="G76" s="19"/>
+      <c r="D76" s="19"/>
+      <c r="G76" s="20"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>45629</v>
       </c>
-      <c r="D77" s="21"/>
-      <c r="G77" s="19"/>
+      <c r="D77" s="19"/>
+      <c r="G77" s="20"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>45630</v>
       </c>
-      <c r="D78" s="21"/>
-      <c r="G78" s="20" t="s">
+      <c r="D78" s="19"/>
+      <c r="G78" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2019,8 +2020,8 @@
       <c r="A79">
         <v>45631</v>
       </c>
-      <c r="D79" s="21"/>
-      <c r="G79" s="20"/>
+      <c r="D79" s="19"/>
+      <c r="G79" s="21"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80">
@@ -2029,16 +2030,16 @@
       <c r="D80" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G80" s="20"/>
+      <c r="G80" s="21"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81">
         <v>45633</v>
       </c>
-      <c r="D81" s="21" t="s">
+      <c r="D81" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G81" s="19" t="s">
+      <c r="G81" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2046,22 +2047,22 @@
       <c r="A82">
         <v>45634</v>
       </c>
-      <c r="D82" s="21"/>
-      <c r="G82" s="19"/>
+      <c r="D82" s="19"/>
+      <c r="G82" s="20"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83">
         <v>45635</v>
       </c>
-      <c r="D83" s="21"/>
-      <c r="G83" s="19"/>
+      <c r="D83" s="19"/>
+      <c r="G83" s="20"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84">
         <v>45636</v>
       </c>
-      <c r="D84" s="21"/>
-      <c r="G84" s="20" t="s">
+      <c r="D84" s="19"/>
+      <c r="G84" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2069,22 +2070,22 @@
       <c r="A85">
         <v>45637</v>
       </c>
-      <c r="D85" s="21"/>
-      <c r="G85" s="20"/>
+      <c r="D85" s="19"/>
+      <c r="G85" s="21"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86">
         <v>45638</v>
       </c>
-      <c r="D86" s="21"/>
-      <c r="G86" s="20"/>
+      <c r="D86" s="19"/>
+      <c r="G86" s="21"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87">
         <v>45639</v>
       </c>
-      <c r="D87" s="21"/>
-      <c r="G87" s="19" t="s">
+      <c r="D87" s="19"/>
+      <c r="G87" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2092,22 +2093,22 @@
       <c r="A88">
         <v>45640</v>
       </c>
-      <c r="D88" s="21"/>
-      <c r="G88" s="19"/>
+      <c r="D88" s="19"/>
+      <c r="G88" s="20"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>45641</v>
       </c>
-      <c r="D89" s="21"/>
-      <c r="G89" s="19"/>
+      <c r="D89" s="19"/>
+      <c r="G89" s="20"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>45642</v>
       </c>
-      <c r="D90" s="21"/>
-      <c r="G90" s="20" t="s">
+      <c r="D90" s="19"/>
+      <c r="G90" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2115,22 +2116,22 @@
       <c r="A91">
         <v>45643</v>
       </c>
-      <c r="D91" s="21"/>
-      <c r="G91" s="20"/>
+      <c r="D91" s="19"/>
+      <c r="G91" s="21"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92">
         <v>45644</v>
       </c>
-      <c r="D92" s="21"/>
-      <c r="G92" s="20"/>
+      <c r="D92" s="19"/>
+      <c r="G92" s="21"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>45645</v>
       </c>
-      <c r="D93" s="21"/>
-      <c r="G93" s="19" t="s">
+      <c r="D93" s="19"/>
+      <c r="G93" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2138,15 +2139,15 @@
       <c r="A94">
         <v>45646</v>
       </c>
-      <c r="D94" s="21"/>
-      <c r="G94" s="19"/>
+      <c r="D94" s="19"/>
+      <c r="G94" s="20"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>45647</v>
       </c>
-      <c r="D95" s="21"/>
-      <c r="G95" s="19"/>
+      <c r="D95" s="19"/>
+      <c r="G95" s="20"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96">
@@ -2165,10 +2166,10 @@
       <c r="A98">
         <v>45792</v>
       </c>
-      <c r="D98" s="21" t="s">
+      <c r="D98" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G98" s="20" t="s">
+      <c r="G98" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2176,22 +2177,22 @@
       <c r="A99">
         <v>45793</v>
       </c>
-      <c r="D99" s="21"/>
-      <c r="G99" s="20"/>
+      <c r="D99" s="19"/>
+      <c r="G99" s="21"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>45794</v>
       </c>
-      <c r="D100" s="21"/>
-      <c r="G100" s="20"/>
+      <c r="D100" s="19"/>
+      <c r="G100" s="21"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>45795</v>
       </c>
-      <c r="D101" s="21"/>
-      <c r="G101" s="19" t="s">
+      <c r="D101" s="19"/>
+      <c r="G101" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2199,22 +2200,22 @@
       <c r="A102">
         <v>45796</v>
       </c>
-      <c r="D102" s="21"/>
-      <c r="G102" s="19"/>
+      <c r="D102" s="19"/>
+      <c r="G102" s="20"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>45797</v>
       </c>
-      <c r="D103" s="21"/>
-      <c r="G103" s="19"/>
+      <c r="D103" s="19"/>
+      <c r="G103" s="20"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>45798</v>
       </c>
-      <c r="D104" s="21"/>
-      <c r="G104" s="20" t="s">
+      <c r="D104" s="19"/>
+      <c r="G104" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2222,22 +2223,22 @@
       <c r="A105">
         <v>45799</v>
       </c>
-      <c r="D105" s="21"/>
-      <c r="G105" s="20"/>
+      <c r="D105" s="19"/>
+      <c r="G105" s="21"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106">
         <v>45800</v>
       </c>
-      <c r="D106" s="21"/>
-      <c r="G106" s="20"/>
+      <c r="D106" s="19"/>
+      <c r="G106" s="21"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107">
         <v>45801</v>
       </c>
-      <c r="D107" s="21"/>
-      <c r="G107" s="19" t="s">
+      <c r="D107" s="19"/>
+      <c r="G107" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2245,22 +2246,22 @@
       <c r="A108">
         <v>45802</v>
       </c>
-      <c r="D108" s="21"/>
-      <c r="G108" s="19"/>
+      <c r="D108" s="19"/>
+      <c r="G108" s="20"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109">
         <v>45803</v>
       </c>
-      <c r="D109" s="21"/>
-      <c r="G109" s="19"/>
+      <c r="D109" s="19"/>
+      <c r="G109" s="20"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A110">
         <v>45804</v>
       </c>
-      <c r="D110" s="21"/>
-      <c r="G110" s="20" t="s">
+      <c r="D110" s="19"/>
+      <c r="G110" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2268,15 +2269,15 @@
       <c r="A111">
         <v>45805</v>
       </c>
-      <c r="D111" s="21"/>
-      <c r="G111" s="20"/>
+      <c r="D111" s="19"/>
+      <c r="G111" s="21"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112">
         <v>45806</v>
       </c>
-      <c r="D112" s="21"/>
-      <c r="G112" s="20"/>
+      <c r="D112" s="19"/>
+      <c r="G112" s="21"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113">
@@ -2285,7 +2286,7 @@
       <c r="D113" t="s">
         <v>28</v>
       </c>
-      <c r="G113" s="19" t="s">
+      <c r="G113" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2293,13 +2294,13 @@
       <c r="A114">
         <v>45808</v>
       </c>
-      <c r="G114" s="19"/>
+      <c r="G114" s="20"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>45809</v>
       </c>
-      <c r="G115" s="19"/>
+      <c r="G115" s="20"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116">
@@ -2330,7 +2331,7 @@
       <c r="A118">
         <v>45812</v>
       </c>
-      <c r="D118" s="21" t="s">
+      <c r="D118" s="19" t="s">
         <v>31</v>
       </c>
       <c r="E118" s="1"/>
@@ -2341,10 +2342,10 @@
       <c r="A119">
         <v>45813</v>
       </c>
-      <c r="D119" s="21"/>
+      <c r="D119" s="19"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
-      <c r="G119" s="19" t="s">
+      <c r="G119" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2352,28 +2353,28 @@
       <c r="A120">
         <v>45814</v>
       </c>
-      <c r="D120" s="21"/>
+      <c r="D120" s="19"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
-      <c r="G120" s="19"/>
+      <c r="G120" s="20"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121">
         <v>45815</v>
       </c>
-      <c r="D121" s="21"/>
+      <c r="D121" s="19"/>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
-      <c r="G121" s="19"/>
+      <c r="G121" s="20"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>45816</v>
       </c>
-      <c r="D122" s="21"/>
+      <c r="D122" s="19"/>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
-      <c r="G122" s="20" t="s">
+      <c r="G122" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2381,28 +2382,28 @@
       <c r="A123">
         <v>45817</v>
       </c>
-      <c r="D123" s="21"/>
+      <c r="D123" s="19"/>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
-      <c r="G123" s="20"/>
+      <c r="G123" s="21"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124">
         <v>45818</v>
       </c>
-      <c r="D124" s="21"/>
+      <c r="D124" s="19"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="20"/>
+      <c r="G124" s="21"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125">
         <v>45819</v>
       </c>
-      <c r="D125" s="21"/>
+      <c r="D125" s="19"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
-      <c r="G125" s="19" t="s">
+      <c r="G125" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2410,28 +2411,28 @@
       <c r="A126">
         <v>45820</v>
       </c>
-      <c r="D126" s="21"/>
+      <c r="D126" s="19"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-      <c r="G126" s="19"/>
+      <c r="G126" s="20"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127">
         <v>45821</v>
       </c>
-      <c r="D127" s="21"/>
+      <c r="D127" s="19"/>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
-      <c r="G127" s="19"/>
+      <c r="G127" s="20"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128">
         <v>45822</v>
       </c>
-      <c r="D128" s="21"/>
+      <c r="D128" s="19"/>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
-      <c r="G128" s="20" t="s">
+      <c r="G128" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2439,28 +2440,28 @@
       <c r="A129">
         <v>45823</v>
       </c>
-      <c r="D129" s="21"/>
+      <c r="D129" s="19"/>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
-      <c r="G129" s="20"/>
+      <c r="G129" s="21"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130">
         <v>45824</v>
       </c>
-      <c r="D130" s="21"/>
+      <c r="D130" s="19"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
-      <c r="G130" s="20"/>
+      <c r="G130" s="21"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131">
         <v>45825</v>
       </c>
-      <c r="D131" s="21"/>
+      <c r="D131" s="19"/>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
-      <c r="G131" s="19" t="s">
+      <c r="G131" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2473,7 +2474,7 @@
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
-      <c r="G132" s="19"/>
+      <c r="G132" s="20"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133">
@@ -2488,12 +2489,48 @@
       <c r="F133" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G133" s="19"/>
+      <c r="G133" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="D5:D18"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="B21:B32"/>
+    <mergeCell ref="B33:B44"/>
+    <mergeCell ref="A45:G47"/>
+    <mergeCell ref="B48:B59"/>
+    <mergeCell ref="G48:G50"/>
+    <mergeCell ref="G51:G53"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="G57:G59"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="G39:G41"/>
+    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="D65:D79"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="G93:G95"/>
+    <mergeCell ref="G98:G100"/>
+    <mergeCell ref="D98:D112"/>
+    <mergeCell ref="G101:G103"/>
+    <mergeCell ref="G104:G106"/>
     <mergeCell ref="D118:D131"/>
-    <mergeCell ref="D5:D18"/>
     <mergeCell ref="G107:G109"/>
     <mergeCell ref="G110:G112"/>
     <mergeCell ref="G113:G115"/>
@@ -2508,42 +2545,6 @@
     <mergeCell ref="G78:G80"/>
     <mergeCell ref="G81:G83"/>
     <mergeCell ref="G84:G86"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="G93:G95"/>
-    <mergeCell ref="G98:G100"/>
-    <mergeCell ref="D98:D112"/>
-    <mergeCell ref="G101:G103"/>
-    <mergeCell ref="G104:G106"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="D65:D79"/>
-    <mergeCell ref="B21:B32"/>
-    <mergeCell ref="B33:B44"/>
-    <mergeCell ref="A45:G47"/>
-    <mergeCell ref="B48:B59"/>
-    <mergeCell ref="G48:G50"/>
-    <mergeCell ref="G51:G53"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="G57:G59"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="G39:G41"/>
-    <mergeCell ref="G42:G44"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
improve timing to reduce dark current
</commit_message>
<xml_diff>
--- a/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
+++ b/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ECC6378-3472-4726-82C1-1DDB88886B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9FE0E7-5C16-4C1B-B648-BF5AC82DAD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="13583" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="64">
   <si>
     <t>SM0</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -258,6 +258,22 @@
   </si>
   <si>
     <t>~15MiB/s</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S3</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S5</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -518,13 +534,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -947,7 +963,7 @@
       <c r="D6" s="19"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -958,7 +974,7 @@
       <c r="D7" s="19"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="20"/>
+      <c r="G7" s="21"/>
       <c r="J7" t="s">
         <v>51</v>
       </c>
@@ -982,7 +998,7 @@
       <c r="D8" s="19"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="20"/>
+      <c r="G8" s="21"/>
       <c r="J8" s="17">
         <v>0</v>
       </c>
@@ -1003,7 +1019,7 @@
       <c r="D9" s="19"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="22" t="s">
         <v>5</v>
       </c>
       <c r="J9">
@@ -1029,7 +1045,7 @@
       <c r="D10" s="19"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="21"/>
+      <c r="G10" s="22"/>
       <c r="J10">
         <v>359</v>
       </c>
@@ -1053,7 +1069,7 @@
       <c r="D11" s="19"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="21"/>
+      <c r="G11" s="22"/>
       <c r="J11">
         <v>1400</v>
       </c>
@@ -1077,7 +1093,7 @@
       <c r="D12" s="19"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="21" t="s">
         <v>6</v>
       </c>
       <c r="J12">
@@ -1103,7 +1119,7 @@
       <c r="D13" s="19"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="20"/>
+      <c r="G13" s="21"/>
       <c r="J13">
         <v>4525</v>
       </c>
@@ -1127,7 +1143,7 @@
       <c r="D14" s="19"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="20"/>
+      <c r="G14" s="21"/>
       <c r="J14">
         <v>6609</v>
       </c>
@@ -1151,7 +1167,7 @@
       <c r="D15" s="19"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="21" t="s">
+      <c r="G15" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1162,7 +1178,7 @@
       <c r="D16" s="19"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="21"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17">
@@ -1171,7 +1187,7 @@
       <c r="D17" s="19"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="21"/>
+      <c r="G17" s="22"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18">
@@ -1180,7 +1196,7 @@
       <c r="D18" s="19"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1193,7 +1209,7 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="20"/>
+      <c r="G19" s="21"/>
     </row>
     <row r="20" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20">
@@ -1208,7 +1224,7 @@
       <c r="F20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G20" s="20"/>
+      <c r="G20" s="21"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21">
@@ -1223,13 +1239,13 @@
       <c r="D21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="20" t="s">
         <v>9</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G21" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1241,10 +1257,12 @@
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="22"/>
+      <c r="D22" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="20"/>
       <c r="F22" s="19"/>
-      <c r="G22" s="21"/>
+      <c r="G22" s="22"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23">
@@ -1255,13 +1273,13 @@
         <v>2</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F23" s="19"/>
-      <c r="G23" s="21"/>
+      <c r="G23" s="22"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24">
@@ -1271,12 +1289,14 @@
       <c r="C24">
         <v>3</v>
       </c>
-      <c r="D24" s="15"/>
+      <c r="D24" s="15" t="s">
+        <v>62</v>
+      </c>
       <c r="E24" s="11"/>
       <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1288,16 +1308,14 @@
       <c r="C25">
         <v>4</v>
       </c>
-      <c r="D25" s="15" t="s">
-        <v>13</v>
-      </c>
+      <c r="D25" s="15"/>
       <c r="E25" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F25" s="22" t="s">
+      <c r="F25" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="20"/>
+      <c r="G25" s="21"/>
     </row>
     <row r="26" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26">
@@ -1310,7 +1328,7 @@
       <c r="D26" s="15"/>
       <c r="E26" s="11"/>
       <c r="F26" s="23"/>
-      <c r="G26" s="20"/>
+      <c r="G26" s="21"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27">
@@ -1321,7 +1339,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>13</v>
@@ -1329,7 +1347,7 @@
       <c r="F27" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="21" t="s">
+      <c r="G27" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H27" t="s">
@@ -1347,7 +1365,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="12"/>
       <c r="F28" s="6"/>
-      <c r="G28" s="21"/>
+      <c r="G28" s="22"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29">
@@ -1362,7 +1380,7 @@
         <v>14</v>
       </c>
       <c r="F29" s="6"/>
-      <c r="G29" s="21"/>
+      <c r="G29" s="22"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30">
@@ -1377,7 +1395,7 @@
       <c r="F30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1390,13 +1408,13 @@
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="8"/>
-      <c r="G31" s="20"/>
+      <c r="G31" s="21"/>
     </row>
     <row r="32" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32">
@@ -1409,7 +1427,7 @@
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
       <c r="F32" s="8"/>
-      <c r="G32" s="20"/>
+      <c r="G32" s="21"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33">
@@ -1430,7 +1448,7 @@
       <c r="F33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H33" t="s">
@@ -1445,10 +1463,12 @@
       <c r="C34">
         <v>1</v>
       </c>
-      <c r="D34" s="14"/>
+      <c r="D34" s="14" t="s">
+        <v>60</v>
+      </c>
       <c r="E34" s="5"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="21"/>
+      <c r="G34" s="22"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35">
@@ -1459,13 +1479,13 @@
         <v>2</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="6"/>
-      <c r="G35" s="21"/>
+      <c r="G35" s="22"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36">
@@ -1475,12 +1495,14 @@
       <c r="C36">
         <v>3</v>
       </c>
-      <c r="D36" s="15"/>
+      <c r="D36" s="15" t="s">
+        <v>62</v>
+      </c>
       <c r="E36" s="11"/>
       <c r="F36" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1492,14 +1514,12 @@
       <c r="C37">
         <v>4</v>
       </c>
-      <c r="D37" s="15" t="s">
-        <v>13</v>
-      </c>
+      <c r="D37" s="15"/>
       <c r="E37" s="11" t="s">
         <v>12</v>
       </c>
       <c r="F37" s="8"/>
-      <c r="G37" s="20"/>
+      <c r="G37" s="21"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A38">
@@ -1512,7 +1532,7 @@
       <c r="D38" s="15"/>
       <c r="E38" s="12"/>
       <c r="F38" s="9"/>
-      <c r="G38" s="20"/>
+      <c r="G38" s="21"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39">
@@ -1523,7 +1543,7 @@
         <v>6</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>13</v>
@@ -1531,7 +1551,7 @@
       <c r="F39" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="21" t="s">
+      <c r="G39" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H39" t="s">
@@ -1549,7 +1569,7 @@
       <c r="D40" s="2"/>
       <c r="E40" s="12"/>
       <c r="F40" s="6"/>
-      <c r="G40" s="21"/>
+      <c r="G40" s="22"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41">
@@ -1564,7 +1584,7 @@
         <v>14</v>
       </c>
       <c r="F41" s="6"/>
-      <c r="G41" s="21"/>
+      <c r="G41" s="22"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42">
@@ -1579,7 +1599,7 @@
       <c r="F42" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="20" t="s">
+      <c r="G42" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1592,13 +1612,13 @@
         <v>10</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="20"/>
+      <c r="G43" s="21"/>
     </row>
     <row r="44" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A44">
@@ -1611,7 +1631,7 @@
       <c r="D44" s="3"/>
       <c r="E44" s="4"/>
       <c r="F44" s="8"/>
-      <c r="G44" s="20"/>
+      <c r="G44" s="21"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A45" s="19" t="s">
@@ -1661,7 +1681,7 @@
       <c r="F48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G48" s="21" t="s">
+      <c r="G48" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H48" t="s">
@@ -1676,10 +1696,12 @@
       <c r="C49">
         <v>1</v>
       </c>
-      <c r="D49" s="14"/>
+      <c r="D49" s="14" t="s">
+        <v>60</v>
+      </c>
       <c r="E49" s="5"/>
       <c r="F49" s="6"/>
-      <c r="G49" s="21"/>
+      <c r="G49" s="22"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A50">
@@ -1690,13 +1712,13 @@
         <v>2</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E50" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F50" s="6"/>
-      <c r="G50" s="21"/>
+      <c r="G50" s="22"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51">
@@ -1706,12 +1728,14 @@
       <c r="C51">
         <v>3</v>
       </c>
-      <c r="D51" s="15"/>
+      <c r="D51" s="15" t="s">
+        <v>62</v>
+      </c>
       <c r="E51" s="11"/>
       <c r="F51" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G51" s="20" t="s">
+      <c r="G51" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1723,14 +1747,12 @@
       <c r="C52">
         <v>4</v>
       </c>
-      <c r="D52" s="15" t="s">
-        <v>13</v>
-      </c>
+      <c r="D52" s="15"/>
       <c r="E52" s="11" t="s">
         <v>12</v>
       </c>
       <c r="F52" s="8"/>
-      <c r="G52" s="20"/>
+      <c r="G52" s="21"/>
     </row>
     <row r="53" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A53">
@@ -1743,7 +1765,7 @@
       <c r="D53" s="15"/>
       <c r="E53" s="12"/>
       <c r="F53" s="9"/>
-      <c r="G53" s="20"/>
+      <c r="G53" s="21"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A54">
@@ -1754,7 +1776,7 @@
         <v>6</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E54" s="12" t="s">
         <v>13</v>
@@ -1762,7 +1784,7 @@
       <c r="F54" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G54" s="21" t="s">
+      <c r="G54" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H54" t="s">
@@ -1780,7 +1802,7 @@
       <c r="D55" s="2"/>
       <c r="E55" s="12"/>
       <c r="F55" s="6"/>
-      <c r="G55" s="21"/>
+      <c r="G55" s="22"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A56">
@@ -1795,7 +1817,7 @@
         <v>14</v>
       </c>
       <c r="F56" s="6"/>
-      <c r="G56" s="21"/>
+      <c r="G56" s="22"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A57">
@@ -1810,7 +1832,7 @@
       <c r="F57" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G57" s="20" t="s">
+      <c r="G57" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1823,13 +1845,13 @@
         <v>10</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F58" s="8"/>
-      <c r="G58" s="20"/>
+      <c r="G58" s="21"/>
     </row>
     <row r="59" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A59">
@@ -1842,7 +1864,7 @@
       <c r="D59" s="3"/>
       <c r="E59" s="4"/>
       <c r="F59" s="8"/>
-      <c r="G59" s="20"/>
+      <c r="G59" s="21"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A60">
@@ -1857,7 +1879,7 @@
       <c r="F60" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G60" s="21" t="s">
+      <c r="G60" s="22" t="s">
         <v>5</v>
       </c>
       <c r="H60" t="s">
@@ -1871,7 +1893,7 @@
       <c r="D61" s="1"/>
       <c r="E61" s="5"/>
       <c r="F61" s="6"/>
-      <c r="G61" s="21"/>
+      <c r="G61" s="22"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A62">
@@ -1881,7 +1903,7 @@
         <v>21</v>
       </c>
       <c r="F62" s="6"/>
-      <c r="G62" s="21"/>
+      <c r="G62" s="22"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A63">
@@ -1891,7 +1913,7 @@
       <c r="F63" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G63" s="20" t="s">
+      <c r="G63" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1903,7 +1925,7 @@
         <v>21</v>
       </c>
       <c r="F64" s="8"/>
-      <c r="G64" s="20"/>
+      <c r="G64" s="21"/>
     </row>
     <row r="65" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A65">
@@ -1913,14 +1935,14 @@
         <v>22</v>
       </c>
       <c r="F65" s="9"/>
-      <c r="G65" s="20"/>
+      <c r="G65" s="21"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>45618</v>
       </c>
       <c r="D66" s="19"/>
-      <c r="G66" s="21" t="s">
+      <c r="G66" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1929,21 +1951,21 @@
         <v>45619</v>
       </c>
       <c r="D67" s="19"/>
-      <c r="G67" s="21"/>
+      <c r="G67" s="22"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>45620</v>
       </c>
       <c r="D68" s="19"/>
-      <c r="G68" s="21"/>
+      <c r="G68" s="22"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>45621</v>
       </c>
       <c r="D69" s="19"/>
-      <c r="G69" s="20" t="s">
+      <c r="G69" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1952,21 +1974,21 @@
         <v>45622</v>
       </c>
       <c r="D70" s="19"/>
-      <c r="G70" s="20"/>
+      <c r="G70" s="21"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>45623</v>
       </c>
       <c r="D71" s="19"/>
-      <c r="G71" s="20"/>
+      <c r="G71" s="21"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>45624</v>
       </c>
       <c r="D72" s="19"/>
-      <c r="G72" s="21" t="s">
+      <c r="G72" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1975,21 +1997,21 @@
         <v>45625</v>
       </c>
       <c r="D73" s="19"/>
-      <c r="G73" s="21"/>
+      <c r="G73" s="22"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>45626</v>
       </c>
       <c r="D74" s="19"/>
-      <c r="G74" s="21"/>
+      <c r="G74" s="22"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>45627</v>
       </c>
       <c r="D75" s="19"/>
-      <c r="G75" s="20" t="s">
+      <c r="G75" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1998,21 +2020,21 @@
         <v>45628</v>
       </c>
       <c r="D76" s="19"/>
-      <c r="G76" s="20"/>
+      <c r="G76" s="21"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>45629</v>
       </c>
       <c r="D77" s="19"/>
-      <c r="G77" s="20"/>
+      <c r="G77" s="21"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>45630</v>
       </c>
       <c r="D78" s="19"/>
-      <c r="G78" s="21" t="s">
+      <c r="G78" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2021,7 +2043,7 @@
         <v>45631</v>
       </c>
       <c r="D79" s="19"/>
-      <c r="G79" s="21"/>
+      <c r="G79" s="22"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80">
@@ -2030,7 +2052,7 @@
       <c r="D80" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G80" s="21"/>
+      <c r="G80" s="22"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81">
@@ -2039,7 +2061,7 @@
       <c r="D81" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G81" s="20" t="s">
+      <c r="G81" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2048,21 +2070,21 @@
         <v>45634</v>
       </c>
       <c r="D82" s="19"/>
-      <c r="G82" s="20"/>
+      <c r="G82" s="21"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83">
         <v>45635</v>
       </c>
       <c r="D83" s="19"/>
-      <c r="G83" s="20"/>
+      <c r="G83" s="21"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84">
         <v>45636</v>
       </c>
       <c r="D84" s="19"/>
-      <c r="G84" s="21" t="s">
+      <c r="G84" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2071,21 +2093,21 @@
         <v>45637</v>
       </c>
       <c r="D85" s="19"/>
-      <c r="G85" s="21"/>
+      <c r="G85" s="22"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86">
         <v>45638</v>
       </c>
       <c r="D86" s="19"/>
-      <c r="G86" s="21"/>
+      <c r="G86" s="22"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87">
         <v>45639</v>
       </c>
       <c r="D87" s="19"/>
-      <c r="G87" s="20" t="s">
+      <c r="G87" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2094,21 +2116,21 @@
         <v>45640</v>
       </c>
       <c r="D88" s="19"/>
-      <c r="G88" s="20"/>
+      <c r="G88" s="21"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>45641</v>
       </c>
       <c r="D89" s="19"/>
-      <c r="G89" s="20"/>
+      <c r="G89" s="21"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>45642</v>
       </c>
       <c r="D90" s="19"/>
-      <c r="G90" s="21" t="s">
+      <c r="G90" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2117,21 +2139,21 @@
         <v>45643</v>
       </c>
       <c r="D91" s="19"/>
-      <c r="G91" s="21"/>
+      <c r="G91" s="22"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92">
         <v>45644</v>
       </c>
       <c r="D92" s="19"/>
-      <c r="G92" s="21"/>
+      <c r="G92" s="22"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>45645</v>
       </c>
       <c r="D93" s="19"/>
-      <c r="G93" s="20" t="s">
+      <c r="G93" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2140,14 +2162,14 @@
         <v>45646</v>
       </c>
       <c r="D94" s="19"/>
-      <c r="G94" s="20"/>
+      <c r="G94" s="21"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>45647</v>
       </c>
       <c r="D95" s="19"/>
-      <c r="G95" s="20"/>
+      <c r="G95" s="21"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96">
@@ -2169,7 +2191,7 @@
       <c r="D98" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G98" s="21" t="s">
+      <c r="G98" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2178,21 +2200,21 @@
         <v>45793</v>
       </c>
       <c r="D99" s="19"/>
-      <c r="G99" s="21"/>
+      <c r="G99" s="22"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>45794</v>
       </c>
       <c r="D100" s="19"/>
-      <c r="G100" s="21"/>
+      <c r="G100" s="22"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>45795</v>
       </c>
       <c r="D101" s="19"/>
-      <c r="G101" s="20" t="s">
+      <c r="G101" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2201,21 +2223,21 @@
         <v>45796</v>
       </c>
       <c r="D102" s="19"/>
-      <c r="G102" s="20"/>
+      <c r="G102" s="21"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>45797</v>
       </c>
       <c r="D103" s="19"/>
-      <c r="G103" s="20"/>
+      <c r="G103" s="21"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>45798</v>
       </c>
       <c r="D104" s="19"/>
-      <c r="G104" s="21" t="s">
+      <c r="G104" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2224,21 +2246,21 @@
         <v>45799</v>
       </c>
       <c r="D105" s="19"/>
-      <c r="G105" s="21"/>
+      <c r="G105" s="22"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106">
         <v>45800</v>
       </c>
       <c r="D106" s="19"/>
-      <c r="G106" s="21"/>
+      <c r="G106" s="22"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107">
         <v>45801</v>
       </c>
       <c r="D107" s="19"/>
-      <c r="G107" s="20" t="s">
+      <c r="G107" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2247,21 +2269,21 @@
         <v>45802</v>
       </c>
       <c r="D108" s="19"/>
-      <c r="G108" s="20"/>
+      <c r="G108" s="21"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109">
         <v>45803</v>
       </c>
       <c r="D109" s="19"/>
-      <c r="G109" s="20"/>
+      <c r="G109" s="21"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A110">
         <v>45804</v>
       </c>
       <c r="D110" s="19"/>
-      <c r="G110" s="21" t="s">
+      <c r="G110" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2270,14 +2292,14 @@
         <v>45805</v>
       </c>
       <c r="D111" s="19"/>
-      <c r="G111" s="21"/>
+      <c r="G111" s="22"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112">
         <v>45806</v>
       </c>
       <c r="D112" s="19"/>
-      <c r="G112" s="21"/>
+      <c r="G112" s="22"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113">
@@ -2286,7 +2308,7 @@
       <c r="D113" t="s">
         <v>28</v>
       </c>
-      <c r="G113" s="20" t="s">
+      <c r="G113" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2294,13 +2316,13 @@
       <c r="A114">
         <v>45808</v>
       </c>
-      <c r="G114" s="20"/>
+      <c r="G114" s="21"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>45809</v>
       </c>
-      <c r="G115" s="20"/>
+      <c r="G115" s="21"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116">
@@ -2345,7 +2367,7 @@
       <c r="D119" s="19"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
-      <c r="G119" s="20" t="s">
+      <c r="G119" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2356,7 +2378,7 @@
       <c r="D120" s="19"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
-      <c r="G120" s="20"/>
+      <c r="G120" s="21"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121">
@@ -2365,7 +2387,7 @@
       <c r="D121" s="19"/>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
-      <c r="G121" s="20"/>
+      <c r="G121" s="21"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122">
@@ -2374,7 +2396,7 @@
       <c r="D122" s="19"/>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
-      <c r="G122" s="21" t="s">
+      <c r="G122" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2385,7 +2407,7 @@
       <c r="D123" s="19"/>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
-      <c r="G123" s="21"/>
+      <c r="G123" s="22"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124">
@@ -2394,7 +2416,7 @@
       <c r="D124" s="19"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="21"/>
+      <c r="G124" s="22"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125">
@@ -2403,7 +2425,7 @@
       <c r="D125" s="19"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
-      <c r="G125" s="20" t="s">
+      <c r="G125" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2414,7 +2436,7 @@
       <c r="D126" s="19"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-      <c r="G126" s="20"/>
+      <c r="G126" s="21"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127">
@@ -2423,7 +2445,7 @@
       <c r="D127" s="19"/>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
-      <c r="G127" s="20"/>
+      <c r="G127" s="21"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128">
@@ -2432,7 +2454,7 @@
       <c r="D128" s="19"/>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
-      <c r="G128" s="21" t="s">
+      <c r="G128" s="22" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2443,7 +2465,7 @@
       <c r="D129" s="19"/>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
-      <c r="G129" s="21"/>
+      <c r="G129" s="22"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130">
@@ -2452,7 +2474,7 @@
       <c r="D130" s="19"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
-      <c r="G130" s="21"/>
+      <c r="G130" s="22"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131">
@@ -2461,7 +2483,7 @@
       <c r="D131" s="19"/>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
-      <c r="G131" s="20" t="s">
+      <c r="G131" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2474,7 +2496,7 @@
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
-      <c r="G132" s="20"/>
+      <c r="G132" s="21"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133">
@@ -2489,20 +2511,37 @@
       <c r="F133" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G133" s="20"/>
+      <c r="G133" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D5:D18"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="D118:D131"/>
+    <mergeCell ref="G107:G109"/>
+    <mergeCell ref="G110:G112"/>
+    <mergeCell ref="G113:G115"/>
+    <mergeCell ref="G119:G121"/>
+    <mergeCell ref="G122:G124"/>
+    <mergeCell ref="G125:G127"/>
+    <mergeCell ref="G128:G130"/>
+    <mergeCell ref="G131:G133"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="G93:G95"/>
+    <mergeCell ref="G98:G100"/>
+    <mergeCell ref="D98:D112"/>
+    <mergeCell ref="G101:G103"/>
+    <mergeCell ref="G104:G106"/>
+    <mergeCell ref="D81:D95"/>
+    <mergeCell ref="G81:G83"/>
+    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="D65:D79"/>
+    <mergeCell ref="G72:G74"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="G78:G80"/>
     <mergeCell ref="B21:B32"/>
     <mergeCell ref="B33:B44"/>
     <mergeCell ref="A45:G47"/>
@@ -2518,33 +2557,16 @@
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="G33:G35"/>
     <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="D65:D79"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="G93:G95"/>
-    <mergeCell ref="G98:G100"/>
-    <mergeCell ref="D98:D112"/>
-    <mergeCell ref="G101:G103"/>
-    <mergeCell ref="G104:G106"/>
-    <mergeCell ref="D118:D131"/>
-    <mergeCell ref="G107:G109"/>
-    <mergeCell ref="G110:G112"/>
-    <mergeCell ref="G113:G115"/>
-    <mergeCell ref="G119:G121"/>
-    <mergeCell ref="G122:G124"/>
-    <mergeCell ref="G125:G127"/>
-    <mergeCell ref="G128:G130"/>
-    <mergeCell ref="G131:G133"/>
-    <mergeCell ref="D81:D95"/>
-    <mergeCell ref="G72:G74"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="G78:G80"/>
-    <mergeCell ref="G81:G83"/>
-    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="D5:D18"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
seperate exposure_ticks with SH delay; allow underclocking; param storage with 2 pages
</commit_message>
<xml_diff>
--- a/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
+++ b/Firmware/Project_PRISM_RP2040/State Machine Sequence.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9FE0E7-5C16-4C1B-B648-BF5AC82DAD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C9D46D-8C49-4A52-ADE9-D5D76887A30B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="13583" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21818" windowHeight="13583" xr2:uid="{F9793F9D-0C99-4FB0-9235-392D105C61DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="62">
   <si>
     <t>SM0</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -86,10 +86,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>S5</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>(irq wait 5)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -125,14 +121,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>delay 12*(x+1)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>suppose X=11, 8*12*(11+1)=1152ns</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>irq wait 5</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -161,30 +149,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>1/2738.3456</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/2000.1280</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/2499.8</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/999.968</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/1250.05</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/1600.1024</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Notes</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -201,22 +165,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>~41MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>~37MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>data rate</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>~30MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Absolute CLK#</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -241,39 +189,83 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>45684 ticks each scan row (exclude expsorure delay)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/2728.30</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>~24MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>~18MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>~15MiB/s</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>S1</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>S2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>S3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>S5</t>
+    <t>out x</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>delay 12*12</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>…</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/2727.6496</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>45827 ticks each scan row (expsorure ticks=0)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>delay 1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>delay 6*(x+1)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>suppose X=0, 8*6*(0+1)=48ns</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/2500.1500</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1999.9860</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1600</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1249.9875</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1000.0240</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/799.9949</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/600.0067</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/499.998</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/320.0016</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/284.7410</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>delay 8</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -281,7 +273,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,15 +300,6 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
@@ -525,22 +508,22 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="7" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -868,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79A0B513-DF69-4CBC-B6AA-CECFB4E17D19}">
-  <dimension ref="A1:N133"/>
+  <dimension ref="A1:M133"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="4" max="4" width="14.6640625" customWidth="1"/>
@@ -880,15 +863,15 @@
     <col min="13" max="13" width="12.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="27.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
-        <v>49</v>
+    <row r="1" spans="1:13" ht="27.75" x14ac:dyDescent="0.4">
+      <c r="A1" s="17" t="s">
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>50</v>
+        <v>24</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -903,33 +886,33 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="D2" s="1"/>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>-18</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>-17</v>
       </c>
@@ -939,279 +922,306 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>-16</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>24</v>
+      <c r="D5" s="20" t="s">
+        <v>23</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="16"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>-15</v>
       </c>
-      <c r="D6" s="19"/>
+      <c r="D6" s="20"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="19" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>-14</v>
       </c>
-      <c r="D7" s="19"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="21"/>
+      <c r="G7" s="19"/>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="K7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="L7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="M7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>-13</v>
       </c>
-      <c r="D8" s="19"/>
+      <c r="D8" s="20"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="21"/>
-      <c r="J8" s="17">
+      <c r="G8" s="19"/>
+      <c r="J8">
         <v>0</v>
       </c>
-      <c r="K8" s="17">
-        <v>45648</v>
-      </c>
-      <c r="L8" s="17">
-        <v>0.36518400000000001</v>
-      </c>
-      <c r="M8" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="K8">
+        <v>45827</v>
+      </c>
+      <c r="L8">
+        <v>0.36666399999999999</v>
+      </c>
+      <c r="M8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>-12</v>
       </c>
-      <c r="D9" s="19"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="21" t="s">
         <v>5</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>695</v>
       </c>
       <c r="K9">
-        <v>45828</v>
+        <v>49997</v>
       </c>
       <c r="L9">
-        <v>0.36652800000000002</v>
+        <v>0.399976</v>
       </c>
       <c r="M9" t="s">
-        <v>56</v>
-      </c>
-      <c r="N9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>-11</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="22"/>
+      <c r="G10" s="21"/>
       <c r="J10">
-        <v>359</v>
+        <v>2779</v>
       </c>
       <c r="K10">
-        <v>50004</v>
+        <v>62501</v>
       </c>
       <c r="L10">
-        <v>0.400032</v>
+        <v>0.50000800000000001</v>
       </c>
       <c r="M10" t="s">
-        <v>37</v>
-      </c>
-      <c r="N10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>-10</v>
       </c>
-      <c r="D11" s="19"/>
+      <c r="D11" s="20"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="22"/>
+      <c r="G11" s="21"/>
       <c r="J11">
-        <v>1400</v>
+        <v>5383</v>
       </c>
       <c r="K11">
-        <v>62496</v>
+        <v>78125</v>
       </c>
       <c r="L11">
-        <v>0.49996800000000002</v>
+        <v>0.625</v>
       </c>
       <c r="M11" t="s">
-        <v>36</v>
-      </c>
-      <c r="N11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>-9</v>
       </c>
-      <c r="D12" s="19"/>
+      <c r="D12" s="20"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="19" t="s">
         <v>6</v>
       </c>
       <c r="J12">
-        <v>2702</v>
+        <v>9029</v>
       </c>
       <c r="K12">
-        <v>78120</v>
+        <v>100001</v>
       </c>
       <c r="L12">
-        <v>0.62495999999999996</v>
+        <v>0.80000800000000005</v>
       </c>
       <c r="M12" t="s">
-        <v>40</v>
-      </c>
-      <c r="N12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>-8</v>
       </c>
-      <c r="D13" s="19"/>
+      <c r="D13" s="20"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="21"/>
+      <c r="G13" s="19"/>
       <c r="J13">
-        <v>4525</v>
+        <v>13195</v>
       </c>
       <c r="K13">
-        <v>99996</v>
+        <v>124997</v>
       </c>
       <c r="L13">
-        <v>0.79996800000000001</v>
+        <v>0.99997599999999998</v>
       </c>
       <c r="M13" t="s">
-        <v>39</v>
-      </c>
-      <c r="N13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>-7</v>
       </c>
-      <c r="D14" s="19"/>
+      <c r="D14" s="20"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="21"/>
+      <c r="G14" s="19"/>
       <c r="J14">
-        <v>6609</v>
+        <v>18404</v>
       </c>
       <c r="K14">
-        <v>125004</v>
+        <v>156251</v>
       </c>
       <c r="L14">
-        <v>1.000032</v>
+        <v>1.250008</v>
       </c>
       <c r="M14" t="s">
-        <v>38</v>
-      </c>
-      <c r="N14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>-6</v>
       </c>
-      <c r="D15" s="19"/>
+      <c r="D15" s="20"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="22" t="s">
+      <c r="G15" s="21" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="J15">
+        <v>27084</v>
+      </c>
+      <c r="K15">
+        <v>208331</v>
+      </c>
+      <c r="L15">
+        <v>1.6666479999999999</v>
+      </c>
+      <c r="M15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>-5</v>
       </c>
-      <c r="D16" s="19"/>
+      <c r="D16" s="20"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="22"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G16" s="21"/>
+      <c r="J16">
+        <v>34029</v>
+      </c>
+      <c r="K16">
+        <v>250001</v>
+      </c>
+      <c r="L16">
+        <v>2.0000079999999998</v>
+      </c>
+      <c r="M16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>-4</v>
       </c>
-      <c r="D17" s="19"/>
+      <c r="D17" s="20"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="22"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G17" s="21"/>
+      <c r="J17">
+        <v>57466</v>
+      </c>
+      <c r="K17">
+        <v>390623</v>
+      </c>
+      <c r="L17">
+        <v>3.124984</v>
+      </c>
+      <c r="M17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>-3</v>
       </c>
-      <c r="D18" s="19"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="21" t="s">
+      <c r="G18" s="19" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="J18">
+        <v>65535</v>
+      </c>
+      <c r="K18">
+        <v>439037</v>
+      </c>
+      <c r="L18">
+        <v>3.5122960000000001</v>
+      </c>
+      <c r="M18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>-2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="21"/>
-    </row>
-    <row r="20" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G19" s="19"/>
+    </row>
+    <row r="20" spans="1:13" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>-1</v>
       </c>
@@ -1224,13 +1234,13 @@
       <c r="F20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G20" s="21"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G20" s="19"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>0</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <v>0</v>
       </c>
       <c r="C21">
@@ -1239,154 +1249,150 @@
       <c r="D21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>1</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="20"/>
       <c r="C22">
         <v>1</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E22" s="20"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="22"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="D22" s="14"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="21"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>2</v>
       </c>
-      <c r="B23" s="19"/>
+      <c r="B23" s="20"/>
       <c r="C23">
         <v>2</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="22"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="F23" s="20"/>
+      <c r="G23" s="21"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>3</v>
       </c>
-      <c r="B24" s="19"/>
+      <c r="B24" s="20"/>
       <c r="C24">
         <v>3</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G24" s="21" t="s">
+      <c r="G24" s="19" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>4</v>
       </c>
-      <c r="B25" s="19"/>
+      <c r="B25" s="20"/>
       <c r="C25">
         <v>4</v>
       </c>
       <c r="D25" s="15"/>
-      <c r="E25" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F25" s="20" t="s">
+      <c r="E25" s="11"/>
+      <c r="F25" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="21"/>
-    </row>
-    <row r="26" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G25" s="19"/>
+    </row>
+    <row r="26" spans="1:13" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>5</v>
       </c>
-      <c r="B26" s="19"/>
+      <c r="B26" s="20"/>
       <c r="C26">
         <v>5</v>
       </c>
       <c r="D26" s="15"/>
-      <c r="E26" s="11"/>
+      <c r="E26" s="11" t="s">
+        <v>42</v>
+      </c>
       <c r="F26" s="23"/>
-      <c r="G26" s="21"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G26" s="19"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>6</v>
       </c>
-      <c r="B27" s="19"/>
+      <c r="B27" s="20"/>
       <c r="C27">
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E27" s="11"/>
       <c r="F27" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H27" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>7</v>
       </c>
-      <c r="B28" s="19"/>
+      <c r="B28" s="20"/>
       <c r="C28">
         <v>7</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="12"/>
       <c r="F28" s="6"/>
-      <c r="G28" s="22"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G28" s="21"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>8</v>
       </c>
-      <c r="B29" s="19"/>
+      <c r="B29" s="20"/>
       <c r="C29">
         <v>8</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F29" s="6"/>
-      <c r="G29" s="22"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="G29" s="21"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>9</v>
       </c>
-      <c r="B30" s="19"/>
+      <c r="B30" s="20"/>
       <c r="C30">
         <v>9</v>
       </c>
@@ -1395,45 +1401,45 @@
       <c r="F30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="21" t="s">
+      <c r="G30" s="19" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>10</v>
       </c>
-      <c r="B31" s="19"/>
+      <c r="B31" s="20"/>
       <c r="C31">
         <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F31" s="8"/>
-      <c r="G31" s="21"/>
-    </row>
-    <row r="32" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G31" s="19"/>
+    </row>
+    <row r="32" spans="1:13" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>11</v>
       </c>
-      <c r="B32" s="19"/>
+      <c r="B32" s="20"/>
       <c r="C32">
         <v>11</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
       <c r="F32" s="8"/>
-      <c r="G32" s="21"/>
+      <c r="G32" s="19"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>12</v>
       </c>
-      <c r="B33" s="19">
+      <c r="B33" s="20">
         <v>1</v>
       </c>
       <c r="C33">
@@ -1443,66 +1449,64 @@
         <v>11</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="22" t="s">
+      <c r="G33" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H33" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>13</v>
       </c>
-      <c r="B34" s="19"/>
+      <c r="B34" s="20"/>
       <c r="C34">
         <v>1</v>
       </c>
-      <c r="D34" s="14" t="s">
-        <v>60</v>
-      </c>
+      <c r="D34" s="14"/>
       <c r="E34" s="5"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="22"/>
+      <c r="G34" s="21"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>14</v>
       </c>
-      <c r="B35" s="19"/>
+      <c r="B35" s="20"/>
       <c r="C35">
         <v>2</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="6"/>
-      <c r="G35" s="22"/>
+      <c r="G35" s="21"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>15</v>
       </c>
-      <c r="B36" s="19"/>
+      <c r="B36" s="20"/>
       <c r="C36">
         <v>3</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="E36" s="11"/>
       <c r="F36" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G36" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1510,87 +1514,85 @@
       <c r="A37">
         <v>16</v>
       </c>
-      <c r="B37" s="19"/>
+      <c r="B37" s="20"/>
       <c r="C37">
         <v>4</v>
       </c>
       <c r="D37" s="15"/>
-      <c r="E37" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="E37" s="11"/>
       <c r="F37" s="8"/>
-      <c r="G37" s="21"/>
+      <c r="G37" s="19"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>17</v>
       </c>
-      <c r="B38" s="19"/>
+      <c r="B38" s="20"/>
       <c r="C38">
         <v>5</v>
       </c>
       <c r="D38" s="15"/>
-      <c r="E38" s="12"/>
+      <c r="E38" s="11" t="s">
+        <v>42</v>
+      </c>
       <c r="F38" s="9"/>
-      <c r="G38" s="21"/>
+      <c r="G38" s="19"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>18</v>
       </c>
-      <c r="B39" s="19"/>
+      <c r="B39" s="20"/>
       <c r="C39">
         <v>6</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E39" s="12" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E39" s="11"/>
       <c r="F39" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="22" t="s">
+      <c r="G39" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H39" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>19</v>
       </c>
-      <c r="B40" s="19"/>
+      <c r="B40" s="20"/>
       <c r="C40">
         <v>7</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="12"/>
       <c r="F40" s="6"/>
-      <c r="G40" s="22"/>
+      <c r="G40" s="21"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>20</v>
       </c>
-      <c r="B41" s="19"/>
+      <c r="B41" s="20"/>
       <c r="C41">
         <v>8</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F41" s="6"/>
-      <c r="G41" s="22"/>
+      <c r="G41" s="21"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>21</v>
       </c>
-      <c r="B42" s="19"/>
+      <c r="B42" s="20"/>
       <c r="C42">
         <v>9</v>
       </c>
@@ -1599,7 +1601,7 @@
       <c r="F42" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="21" t="s">
+      <c r="G42" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1607,66 +1609,66 @@
       <c r="A43">
         <v>22</v>
       </c>
-      <c r="B43" s="19"/>
+      <c r="B43" s="20"/>
       <c r="C43">
         <v>10</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="21"/>
+      <c r="G43" s="19"/>
     </row>
     <row r="44" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>23</v>
       </c>
-      <c r="B44" s="19"/>
+      <c r="B44" s="20"/>
       <c r="C44">
         <v>11</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="4"/>
       <c r="F44" s="8"/>
-      <c r="G44" s="21"/>
+      <c r="G44" s="19"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A45" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
+      <c r="A45" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
     </row>
     <row r="47" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="19"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>45600</v>
       </c>
-      <c r="B48" s="19">
+      <c r="B48" s="20">
         <v>3800</v>
       </c>
       <c r="C48">
@@ -1676,66 +1678,64 @@
         <v>11</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G48" s="22" t="s">
+      <c r="G48" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H48" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>45601</v>
       </c>
-      <c r="B49" s="19"/>
+      <c r="B49" s="20"/>
       <c r="C49">
         <v>1</v>
       </c>
-      <c r="D49" s="14" t="s">
-        <v>60</v>
-      </c>
+      <c r="D49" s="14"/>
       <c r="E49" s="5"/>
       <c r="F49" s="6"/>
-      <c r="G49" s="22"/>
+      <c r="G49" s="21"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>45602</v>
       </c>
-      <c r="B50" s="19"/>
+      <c r="B50" s="20"/>
       <c r="C50">
         <v>2</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E50" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F50" s="6"/>
-      <c r="G50" s="22"/>
+      <c r="G50" s="21"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>45603</v>
       </c>
-      <c r="B51" s="19"/>
+      <c r="B51" s="20"/>
       <c r="C51">
         <v>3</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="E51" s="11"/>
       <c r="F51" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G51" s="21" t="s">
+      <c r="G51" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1743,87 +1743,85 @@
       <c r="A52">
         <v>45604</v>
       </c>
-      <c r="B52" s="19"/>
+      <c r="B52" s="20"/>
       <c r="C52">
         <v>4</v>
       </c>
       <c r="D52" s="15"/>
-      <c r="E52" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="E52" s="11"/>
       <c r="F52" s="8"/>
-      <c r="G52" s="21"/>
+      <c r="G52" s="19"/>
     </row>
     <row r="53" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>45605</v>
       </c>
-      <c r="B53" s="19"/>
+      <c r="B53" s="20"/>
       <c r="C53">
         <v>5</v>
       </c>
       <c r="D53" s="15"/>
-      <c r="E53" s="12"/>
+      <c r="E53" s="11" t="s">
+        <v>42</v>
+      </c>
       <c r="F53" s="9"/>
-      <c r="G53" s="21"/>
+      <c r="G53" s="19"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>45606</v>
       </c>
-      <c r="B54" s="19"/>
+      <c r="B54" s="20"/>
       <c r="C54">
         <v>6</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E54" s="12" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E54" s="11"/>
       <c r="F54" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G54" s="22" t="s">
+      <c r="G54" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H54" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>45607</v>
       </c>
-      <c r="B55" s="19"/>
+      <c r="B55" s="20"/>
       <c r="C55">
         <v>7</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="12"/>
       <c r="F55" s="6"/>
-      <c r="G55" s="22"/>
+      <c r="G55" s="21"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>45608</v>
       </c>
-      <c r="B56" s="19"/>
+      <c r="B56" s="20"/>
       <c r="C56">
         <v>8</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F56" s="6"/>
-      <c r="G56" s="22"/>
+      <c r="G56" s="21"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>45609</v>
       </c>
-      <c r="B57" s="19"/>
+      <c r="B57" s="20"/>
       <c r="C57">
         <v>9</v>
       </c>
@@ -1832,7 +1830,7 @@
       <c r="F57" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G57" s="21" t="s">
+      <c r="G57" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1840,80 +1838,84 @@
       <c r="A58">
         <v>45610</v>
       </c>
-      <c r="B58" s="19"/>
+      <c r="B58" s="20"/>
       <c r="C58">
         <v>10</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F58" s="8"/>
-      <c r="G58" s="21"/>
+      <c r="G58" s="19"/>
     </row>
     <row r="59" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>45611</v>
       </c>
-      <c r="B59" s="19"/>
+      <c r="B59" s="20"/>
       <c r="C59">
         <v>11</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="4"/>
       <c r="F59" s="8"/>
-      <c r="G59" s="21"/>
+      <c r="G59" s="19"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A60">
         <v>45612</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G60" s="22" t="s">
+      <c r="G60" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H60" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>45613</v>
       </c>
-      <c r="D61" s="1"/>
+      <c r="D61" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="E61" s="5"/>
       <c r="F61" s="6"/>
-      <c r="G61" s="22"/>
+      <c r="G61" s="21"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>45614</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F62" s="6"/>
-      <c r="G62" s="22"/>
+      <c r="G62" s="21"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A63">
         <v>45615</v>
       </c>
-      <c r="D63" s="1"/>
+      <c r="D63" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="F63" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G63" s="21" t="s">
+      <c r="G63" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1922,27 +1924,27 @@
         <v>45616</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F64" s="8"/>
-      <c r="G64" s="21"/>
+      <c r="G64" s="19"/>
     </row>
     <row r="65" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>45617</v>
       </c>
-      <c r="D65" s="19" t="s">
-        <v>22</v>
+      <c r="D65" s="20" t="s">
+        <v>21</v>
       </c>
       <c r="F65" s="9"/>
-      <c r="G65" s="21"/>
+      <c r="G65" s="19"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>45618</v>
       </c>
-      <c r="D66" s="19"/>
-      <c r="G66" s="22" t="s">
+      <c r="D66" s="20"/>
+      <c r="G66" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1950,22 +1952,22 @@
       <c r="A67">
         <v>45619</v>
       </c>
-      <c r="D67" s="19"/>
-      <c r="G67" s="22"/>
+      <c r="D67" s="20"/>
+      <c r="G67" s="21"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>45620</v>
       </c>
-      <c r="D68" s="19"/>
-      <c r="G68" s="22"/>
+      <c r="D68" s="20"/>
+      <c r="G68" s="21"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>45621</v>
       </c>
-      <c r="D69" s="19"/>
-      <c r="G69" s="21" t="s">
+      <c r="D69" s="20"/>
+      <c r="G69" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1973,22 +1975,22 @@
       <c r="A70">
         <v>45622</v>
       </c>
-      <c r="D70" s="19"/>
-      <c r="G70" s="21"/>
+      <c r="D70" s="20"/>
+      <c r="G70" s="19"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>45623</v>
       </c>
-      <c r="D71" s="19"/>
-      <c r="G71" s="21"/>
+      <c r="D71" s="20"/>
+      <c r="G71" s="19"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>45624</v>
       </c>
-      <c r="D72" s="19"/>
-      <c r="G72" s="22" t="s">
+      <c r="D72" s="20"/>
+      <c r="G72" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1996,22 +1998,22 @@
       <c r="A73">
         <v>45625</v>
       </c>
-      <c r="D73" s="19"/>
-      <c r="G73" s="22"/>
+      <c r="D73" s="20"/>
+      <c r="G73" s="21"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>45626</v>
       </c>
-      <c r="D74" s="19"/>
-      <c r="G74" s="22"/>
+      <c r="D74" s="20"/>
+      <c r="G74" s="21"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>45627</v>
       </c>
-      <c r="D75" s="19"/>
-      <c r="G75" s="21" t="s">
+      <c r="D75" s="20"/>
+      <c r="G75" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2019,22 +2021,22 @@
       <c r="A76">
         <v>45628</v>
       </c>
-      <c r="D76" s="19"/>
-      <c r="G76" s="21"/>
+      <c r="D76" s="20"/>
+      <c r="G76" s="19"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>45629</v>
       </c>
-      <c r="D77" s="19"/>
-      <c r="G77" s="21"/>
+      <c r="D77" s="20"/>
+      <c r="G77" s="19"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>45630</v>
       </c>
-      <c r="D78" s="19"/>
-      <c r="G78" s="22" t="s">
+      <c r="D78" s="20"/>
+      <c r="G78" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2042,26 +2044,26 @@
       <c r="A79">
         <v>45631</v>
       </c>
-      <c r="D79" s="19"/>
-      <c r="G79" s="22"/>
+      <c r="D79" s="20"/>
+      <c r="G79" s="21"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80">
         <v>45632</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G80" s="22"/>
+        <v>22</v>
+      </c>
+      <c r="G80" s="21"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81">
         <v>45633</v>
       </c>
-      <c r="D81" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G81" s="21" t="s">
+      <c r="D81" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="G81" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2069,22 +2071,22 @@
       <c r="A82">
         <v>45634</v>
       </c>
-      <c r="D82" s="19"/>
-      <c r="G82" s="21"/>
+      <c r="D82" s="20"/>
+      <c r="G82" s="19"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83">
         <v>45635</v>
       </c>
-      <c r="D83" s="19"/>
-      <c r="G83" s="21"/>
+      <c r="D83" s="20"/>
+      <c r="G83" s="19"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84">
         <v>45636</v>
       </c>
-      <c r="D84" s="19"/>
-      <c r="G84" s="22" t="s">
+      <c r="D84" s="20"/>
+      <c r="G84" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2092,22 +2094,22 @@
       <c r="A85">
         <v>45637</v>
       </c>
-      <c r="D85" s="19"/>
-      <c r="G85" s="22"/>
+      <c r="D85" s="20"/>
+      <c r="G85" s="21"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86">
         <v>45638</v>
       </c>
-      <c r="D86" s="19"/>
-      <c r="G86" s="22"/>
+      <c r="D86" s="20"/>
+      <c r="G86" s="21"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87">
         <v>45639</v>
       </c>
-      <c r="D87" s="19"/>
-      <c r="G87" s="21" t="s">
+      <c r="D87" s="20"/>
+      <c r="G87" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2115,22 +2117,26 @@
       <c r="A88">
         <v>45640</v>
       </c>
-      <c r="D88" s="19"/>
-      <c r="G88" s="21"/>
+      <c r="D88" s="20"/>
+      <c r="G88" s="19"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>45641</v>
       </c>
-      <c r="D89" s="19"/>
-      <c r="G89" s="21"/>
+      <c r="D89" t="s">
+        <v>49</v>
+      </c>
+      <c r="G89" s="19"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>45642</v>
       </c>
-      <c r="D90" s="19"/>
-      <c r="G90" s="22" t="s">
+      <c r="D90" t="s">
+        <v>50</v>
+      </c>
+      <c r="G90" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2138,22 +2144,19 @@
       <c r="A91">
         <v>45643</v>
       </c>
-      <c r="D91" s="19"/>
-      <c r="G91" s="22"/>
+      <c r="G91" s="21"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92">
         <v>45644</v>
       </c>
-      <c r="D92" s="19"/>
-      <c r="G92" s="22"/>
+      <c r="G92" s="21"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>45645</v>
       </c>
-      <c r="D93" s="19"/>
-      <c r="G93" s="21" t="s">
+      <c r="G93" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2161,37 +2164,44 @@
       <c r="A94">
         <v>45646</v>
       </c>
-      <c r="D94" s="19"/>
-      <c r="G94" s="21"/>
+      <c r="G94" s="19"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>45647</v>
       </c>
-      <c r="D95" s="19"/>
-      <c r="G95" s="21"/>
+      <c r="D95" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G95" s="19"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96">
         <v>45648</v>
       </c>
-      <c r="D96" t="s">
-        <v>26</v>
+      <c r="D96" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G96" s="16" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="D97" t="s">
-        <v>27</v>
+      <c r="A97" t="s">
+        <v>45</v>
+      </c>
+      <c r="G97" s="18" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>45792</v>
       </c>
-      <c r="D98" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G98" s="22" t="s">
+      <c r="D98" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G98" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2199,22 +2209,24 @@
       <c r="A99">
         <v>45793</v>
       </c>
-      <c r="D99" s="19"/>
-      <c r="G99" s="22"/>
+      <c r="D99" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G99" s="21"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>45794</v>
       </c>
-      <c r="D100" s="19"/>
-      <c r="G100" s="22"/>
+      <c r="D100" s="20"/>
+      <c r="G100" s="21"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>45795</v>
       </c>
-      <c r="D101" s="19"/>
-      <c r="G101" s="21" t="s">
+      <c r="D101" s="20"/>
+      <c r="G101" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2222,22 +2234,22 @@
       <c r="A102">
         <v>45796</v>
       </c>
-      <c r="D102" s="19"/>
-      <c r="G102" s="21"/>
+      <c r="D102" s="20"/>
+      <c r="G102" s="19"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>45797</v>
       </c>
-      <c r="D103" s="19"/>
-      <c r="G103" s="21"/>
+      <c r="D103" s="20"/>
+      <c r="G103" s="19"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>45798</v>
       </c>
-      <c r="D104" s="19"/>
-      <c r="G104" s="22" t="s">
+      <c r="D104" s="20"/>
+      <c r="G104" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2245,22 +2257,22 @@
       <c r="A105">
         <v>45799</v>
       </c>
-      <c r="D105" s="19"/>
-      <c r="G105" s="22"/>
+      <c r="D105" s="20"/>
+      <c r="G105" s="21"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106">
         <v>45800</v>
       </c>
-      <c r="D106" s="19"/>
-      <c r="G106" s="22"/>
+      <c r="D106" s="20"/>
+      <c r="G106" s="21"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107">
         <v>45801</v>
       </c>
-      <c r="D107" s="19"/>
-      <c r="G107" s="21" t="s">
+      <c r="D107" s="20"/>
+      <c r="G107" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2268,22 +2280,22 @@
       <c r="A108">
         <v>45802</v>
       </c>
-      <c r="D108" s="19"/>
-      <c r="G108" s="21"/>
+      <c r="D108" s="20"/>
+      <c r="G108" s="19"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109">
         <v>45803</v>
       </c>
-      <c r="D109" s="19"/>
-      <c r="G109" s="21"/>
+      <c r="D109" s="20"/>
+      <c r="G109" s="19"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A110">
         <v>45804</v>
       </c>
-      <c r="D110" s="19"/>
-      <c r="G110" s="22" t="s">
+      <c r="D110" s="20"/>
+      <c r="G110" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2291,24 +2303,22 @@
       <c r="A111">
         <v>45805</v>
       </c>
-      <c r="D111" s="19"/>
-      <c r="G111" s="22"/>
+      <c r="D111" s="20"/>
+      <c r="G111" s="21"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112">
         <v>45806</v>
       </c>
-      <c r="D112" s="19"/>
-      <c r="G112" s="22"/>
+      <c r="D112" s="20"/>
+      <c r="G112" s="21"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113">
         <v>45807</v>
       </c>
-      <c r="D113" t="s">
-        <v>28</v>
-      </c>
-      <c r="G113" s="21" t="s">
+      <c r="D113" s="20"/>
+      <c r="G113" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2316,24 +2326,27 @@
       <c r="A114">
         <v>45808</v>
       </c>
-      <c r="G114" s="21"/>
+      <c r="D114" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G114" s="19"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>45809</v>
       </c>
-      <c r="G115" s="21"/>
+      <c r="G115" s="19"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116">
         <v>45810</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E116" s="1"/>
       <c r="G116" s="16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.4">
@@ -2346,15 +2359,15 @@
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>45812</v>
       </c>
-      <c r="D118" s="19" t="s">
-        <v>31</v>
+      <c r="D118" s="20" t="s">
+        <v>28</v>
       </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
@@ -2364,10 +2377,10 @@
       <c r="A119">
         <v>45813</v>
       </c>
-      <c r="D119" s="19"/>
+      <c r="D119" s="20"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
-      <c r="G119" s="21" t="s">
+      <c r="G119" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2375,28 +2388,28 @@
       <c r="A120">
         <v>45814</v>
       </c>
-      <c r="D120" s="19"/>
+      <c r="D120" s="20"/>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
-      <c r="G120" s="21"/>
+      <c r="G120" s="19"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121">
         <v>45815</v>
       </c>
-      <c r="D121" s="19"/>
+      <c r="D121" s="20"/>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
-      <c r="G121" s="21"/>
+      <c r="G121" s="19"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>45816</v>
       </c>
-      <c r="D122" s="19"/>
+      <c r="D122" s="20"/>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
-      <c r="G122" s="22" t="s">
+      <c r="G122" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2404,28 +2417,28 @@
       <c r="A123">
         <v>45817</v>
       </c>
-      <c r="D123" s="19"/>
+      <c r="D123" s="20"/>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
-      <c r="G123" s="22"/>
+      <c r="G123" s="21"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124">
         <v>45818</v>
       </c>
-      <c r="D124" s="19"/>
+      <c r="D124" s="20"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="22"/>
+      <c r="G124" s="21"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125">
         <v>45819</v>
       </c>
-      <c r="D125" s="19"/>
+      <c r="D125" s="20"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
-      <c r="G125" s="21" t="s">
+      <c r="G125" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2433,28 +2446,28 @@
       <c r="A126">
         <v>45820</v>
       </c>
-      <c r="D126" s="19"/>
+      <c r="D126" s="20"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-      <c r="G126" s="21"/>
+      <c r="G126" s="19"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127">
         <v>45821</v>
       </c>
-      <c r="D127" s="19"/>
+      <c r="D127" s="20"/>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
-      <c r="G127" s="21"/>
+      <c r="G127" s="19"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128">
         <v>45822</v>
       </c>
-      <c r="D128" s="19"/>
+      <c r="D128" s="20"/>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
-      <c r="G128" s="22" t="s">
+      <c r="G128" s="21" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2462,28 +2475,28 @@
       <c r="A129">
         <v>45823</v>
       </c>
-      <c r="D129" s="19"/>
+      <c r="D129" s="20"/>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
-      <c r="G129" s="22"/>
+      <c r="G129" s="21"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130">
         <v>45824</v>
       </c>
-      <c r="D130" s="19"/>
+      <c r="D130" s="20"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
-      <c r="G130" s="22"/>
+      <c r="G130" s="21"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131">
         <v>45825</v>
       </c>
-      <c r="D131" s="19"/>
+      <c r="D131" s="20"/>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
-      <c r="G131" s="21" t="s">
+      <c r="G131" s="19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2492,11 +2505,11 @@
         <v>45826</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
-      <c r="G132" s="21"/>
+      <c r="G132" s="19"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133">
@@ -2511,37 +2524,23 @@
       <c r="F133" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G133" s="21"/>
+      <c r="G133" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D118:D131"/>
-    <mergeCell ref="G107:G109"/>
-    <mergeCell ref="G110:G112"/>
-    <mergeCell ref="G113:G115"/>
-    <mergeCell ref="G119:G121"/>
-    <mergeCell ref="G122:G124"/>
-    <mergeCell ref="G125:G127"/>
-    <mergeCell ref="G128:G130"/>
-    <mergeCell ref="G131:G133"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="G93:G95"/>
     <mergeCell ref="G98:G100"/>
-    <mergeCell ref="D98:D112"/>
     <mergeCell ref="G101:G103"/>
     <mergeCell ref="G104:G106"/>
-    <mergeCell ref="D81:D95"/>
-    <mergeCell ref="G81:G83"/>
-    <mergeCell ref="G84:G86"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="D65:D79"/>
-    <mergeCell ref="G72:G74"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="D5:D18"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="B21:B32"/>
     <mergeCell ref="B33:B44"/>
     <mergeCell ref="A45:G47"/>
@@ -2557,16 +2556,30 @@
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="G33:G35"/>
     <mergeCell ref="G27:G29"/>
-    <mergeCell ref="D5:D18"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="D65:D79"/>
+    <mergeCell ref="G72:G74"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="G81:G83"/>
+    <mergeCell ref="D118:D131"/>
+    <mergeCell ref="G107:G109"/>
+    <mergeCell ref="G119:G121"/>
+    <mergeCell ref="G122:G124"/>
+    <mergeCell ref="G125:G127"/>
+    <mergeCell ref="G128:G130"/>
+    <mergeCell ref="G131:G133"/>
+    <mergeCell ref="G113:G115"/>
+    <mergeCell ref="G110:G112"/>
+    <mergeCell ref="D81:D88"/>
+    <mergeCell ref="D99:D113"/>
+    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="G93:G95"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>